<commit_message>
Skladová karta: druhý list pro duplex, pořadí odkazů na práci.
Excel export až 80 řádků deníku (40+40 na dvou listech), šablona se stranou 2; na práci nejdřív Plná karta, pak náhled skladové karty.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/deploy/excel/skladova-karta.template.xlsx
+++ b/deploy/excel/skladova-karta.template.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xml:space="preserve">
   <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
-  <workbookPr defaultThemeVersion="124226"/>
+  <workbookPr codeName="ThisWorkbook"/>
   <bookViews>
-    <workbookView xWindow="120" yWindow="90" windowWidth="25815" windowHeight="11010"/>
+    <workbookView activeTab="0" autoFilterDateGrouping="true" firstSheet="0" minimized="false" showHorizontalScroll="true" showSheetTabs="true" showVerticalScroll="true" tabRatio="600" visibility="visible"/>
   </bookViews>
   <sheets>
-    <sheet name="Лист1" sheetId="1" r:id="rId1"/>
-    <sheet name="Лист2" sheetId="2" r:id="rId2"/>
-    <sheet name="Лист3" sheetId="3" r:id="rId3"/>
+    <sheet name="Strana 1" sheetId="1" r:id="rId4"/>
+    <sheet name="Strana 2" sheetId="2" r:id="rId5"/>
   </sheets>
-  <calcPr calcId="124519"/>
+  <definedNames/>
+  <calcPr calcId="999999" calcMode="auto" calcCompleted="1" fullCalcOnLoad="0" forceFullCalc="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="15">
   <si>
     <t>SKLADOVÁ KARTA - OPTIKA</t>
   </si>
@@ -24,19 +24,10 @@
     <t>DATUM NASKLADNĚNÍ :</t>
   </si>
   <si>
-    <t>CELKOVÁ METRÁŽ</t>
-  </si>
-  <si>
     <t>POČET VLÁKEN:</t>
   </si>
   <si>
-    <t>POČÁTEČNÍ STAV</t>
-  </si>
-  <si>
-    <t>TYP OK:</t>
-  </si>
-  <si>
-    <t>POZNÁMKA:</t>
+    <t>4 vl</t>
   </si>
   <si>
     <t>ŠARŽE:</t>
@@ -45,35 +36,45 @@
     <t>450-020858</t>
   </si>
   <si>
+    <t>TYP OK:</t>
+  </si>
+  <si>
     <r>
       <t xml:space="preserve">MLT  DROP  </t>
     </r>
     <r>
       <rPr>
-        <u/>
+        <rFont val="Calibri"/>
+        <b val="false"/>
+        <i val="false"/>
+        <strike val="false"/>
+        <color rgb="FF000000"/>
         <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="minor"/>
+        <u val="single"/>
       </rPr>
-      <t>BLOWN</t>
+      <t xml:space="preserve">BLOWN</t>
     </r>
     <r>
       <rPr>
+        <rFont val="Calibri"/>
+        <b val="false"/>
+        <i val="false"/>
+        <strike val="false"/>
+        <color rgb="FF000000"/>
         <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="minor"/>
+        <u val="none"/>
       </rPr>
       <t xml:space="preserve">  FLAT</t>
     </r>
   </si>
   <si>
-    <t>4 vl</t>
+    <t>CELKOVÁ METRÁŽ</t>
+  </si>
+  <si>
+    <t>POČÁTEČNÍ STAV</t>
+  </si>
+  <si>
+    <t>POZNÁMKA:</t>
   </si>
   <si>
     <t>DATUM</t>
@@ -91,103 +92,80 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xml:space="preserve">
   <numFmts count="2">
-    <numFmt numFmtId="44" formatCode="_-* #,##0.00\ &quot;₴&quot;_-;\-* #,##0.00\ &quot;₴&quot;_-;_-* &quot;-&quot;??\ &quot;₴&quot;_-;_-@_-"/>
-    <numFmt numFmtId="164" formatCode="#,##0.0\ _₴"/>
+    <numFmt numFmtId="164" formatCode="_-* #,##0.00\ &quot;₴&quot;_-;\-* #,##0.00\ &quot;₴&quot;_-;_-* &quot;-&quot;??\ &quot;₴&quot;_-;_-@_-"/>
+    <numFmt numFmtId="165" formatCode="#,##0.0\ _₴"/>
   </numFmts>
-  <fonts count="11">
+  <fonts count="7">
     <font>
+      <b val="0"/>
+      <i val="0"/>
+      <strike val="0"/>
+      <u val="none"/>
       <sz val="11"/>
-      <color theme="1"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
-      <family val="2"/>
-      <charset val="1"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
+      <b val="1"/>
+      <i val="0"/>
+      <strike val="0"/>
+      <u val="none"/>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
-      <family val="2"/>
-      <charset val="1"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="18"/>
-      <color theme="1"/>
+      <b val="1"/>
+      <i val="0"/>
+      <strike val="0"/>
+      <u val="none"/>
+      <sz val="20"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
-      <family val="2"/>
-      <charset val="204"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="20"/>
-      <color theme="1"/>
+      <b val="1"/>
+      <i val="0"/>
+      <strike val="0"/>
+      <u val="none"/>
+      <sz val="18"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
-      <family val="2"/>
-      <charset val="204"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
+      <b val="1"/>
+      <i val="0"/>
+      <strike val="0"/>
+      <u val="none"/>
       <sz val="22"/>
-      <color theme="1"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
-      <family val="2"/>
-      <charset val="204"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="12"/>
-      <color theme="1"/>
+      <b val="0"/>
+      <i val="0"/>
+      <strike val="0"/>
+      <u val="none"/>
+      <sz val="13"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
-      <family val="2"/>
-      <charset val="204"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
+      <b val="0"/>
+      <i val="0"/>
+      <strike val="0"/>
+      <u val="none"/>
+      <sz val="14"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
-      <family val="2"/>
-      <charset val="204"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <charset val="204"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="13"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <charset val="204"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="14"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <charset val="204"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="14"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <charset val="1"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -200,8 +178,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="0" tint="-0.249977111117893"/>
-        <bgColor indexed="64"/>
+        <fgColor rgb="FFBFBFBF"/>
+        <bgColor rgb="FFFFFFFF"/>
       </patternFill>
     </fill>
   </fills>
@@ -214,12 +192,87 @@
       <diagonal/>
     </border>
     <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
       <left style="thin">
-        <color indexed="64"/>
+        <color rgb="FF000000"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
       </left>
       <right/>
       <top style="thin">
-        <color indexed="64"/>
+        <color rgb="FF000000"/>
       </top>
       <bottom/>
       <diagonal/>
@@ -228,7 +281,7 @@
       <left/>
       <right/>
       <top style="thin">
-        <color indexed="64"/>
+        <color rgb="FF000000"/>
       </top>
       <bottom/>
       <diagonal/>
@@ -236,229 +289,152 @@
     <border>
       <left/>
       <right style="thin">
-        <color indexed="64"/>
+        <color rgb="FF000000"/>
       </right>
       <top style="thin">
-        <color indexed="64"/>
+        <color rgb="FF000000"/>
       </top>
       <bottom/>
       <diagonal/>
     </border>
     <border>
       <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
+        <color rgb="FF000000"/>
       </left>
       <right/>
       <top style="thin">
-        <color indexed="64"/>
+        <color rgb="FF000000"/>
       </top>
       <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
+        <color rgb="FF000000"/>
       </bottom>
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="41">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
-    <xf numFmtId="14" fontId="2" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="2" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="0" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
+    <xf xfId="0" fontId="0" numFmtId="164" fillId="0" borderId="0" applyFont="0" applyNumberFormat="1" applyFill="0" applyBorder="0" applyAlignment="0"/>
+    <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="0" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
+    <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="1" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="0"/>
+    <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="2" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="0"/>
+    <xf xfId="0" fontId="1" numFmtId="0" fillId="0" borderId="1" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="1" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="2" numFmtId="0" fillId="0" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="2" numFmtId="0" fillId="0" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="1">
+      <alignment vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="2" numFmtId="0" fillId="0" borderId="2" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="3" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="0"/>
+    <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="4" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="0"/>
+    <xf xfId="0" fontId="3" numFmtId="14" fillId="0" borderId="1" applyFont="1" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="3" numFmtId="14" fillId="0" borderId="2" applyFont="1" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="2" numFmtId="165" fillId="0" borderId="5" applyFont="1" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="2" numFmtId="165" fillId="0" borderId="6" applyFont="1" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="2" numFmtId="165" fillId="0" borderId="7" applyFont="1" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="3" numFmtId="0" fillId="0" borderId="5" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="3" numFmtId="0" fillId="0" borderId="7" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="2" numFmtId="0" fillId="0" borderId="5" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="2" numFmtId="0" fillId="0" borderId="6" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="2" numFmtId="0" fillId="0" borderId="7" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="2" numFmtId="0" fillId="0" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="4" numFmtId="164" fillId="0" borderId="0" applyFont="1" applyNumberFormat="1" applyFill="0" applyBorder="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="8" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="9" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="10" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="4" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="0" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="0" numFmtId="0" fillId="2" borderId="4" applyFont="0" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="0" numFmtId="0" fillId="2" borderId="0" applyFont="0" applyNumberFormat="0" applyFill="1" applyBorder="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="5" numFmtId="0" fillId="0" borderId="11" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="5" numFmtId="0" fillId="0" borderId="5" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="5" numFmtId="0" fillId="0" borderId="8" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="5" numFmtId="0" fillId="0" borderId="10" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="5" numFmtId="0" fillId="0" borderId="11" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="5" numFmtId="0" fillId="0" borderId="9" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="6" numFmtId="0" fillId="2" borderId="4" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="6" numFmtId="0" fillId="2" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="6" numFmtId="0" fillId="2" borderId="4" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="6" numFmtId="0" fillId="2" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
     </xf>
   </cellXfs>
-  <cellStyles count="2">
-    <cellStyle name="Денежный" xfId="1" builtinId="4"/>
-    <cellStyle name="Обычный" xfId="0" builtinId="0"/>
+  <cellStyles count="1">
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <tableStyles defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotTableStyle1"/>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Тема Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Стандартная">
       <a:dk1>
@@ -568,7 +544,7 @@
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Стандартная">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -741,22 +717,25 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xml:space="preserve" mc:Ignorable="x14ac">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+  </sheetPr>
   <dimension ref="A1:L48"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col min="1" max="1" width="9.28515625" customWidth="1"/>
-    <col min="2" max="2" width="10.28515625" customWidth="1"/>
-    <col min="4" max="4" width="13" customWidth="1"/>
-    <col min="5" max="5" width="7.28515625" customWidth="1"/>
-    <col min="6" max="6" width="9.28515625" customWidth="1"/>
-    <col min="7" max="7" width="6.7109375" customWidth="1"/>
-    <col min="8" max="8" width="6.85546875" customWidth="1"/>
-    <col min="9" max="9" width="16.42578125" customWidth="1"/>
-    <col min="10" max="10" width="1" customWidth="1"/>
+    <col min="1" max="1" width="9.28515625" customWidth="true" style="0"/>
+    <col min="2" max="2" width="10.28515625" customWidth="true" style="0"/>
+    <col min="4" max="4" width="13" customWidth="true" style="0"/>
+    <col min="5" max="5" width="7.28515625" customWidth="true" style="0"/>
+    <col min="6" max="6" width="9.28515625" customWidth="true" style="0"/>
+    <col min="7" max="7" width="6.7109375" customWidth="true" style="0"/>
+    <col min="8" max="8" width="6.85546875" customWidth="true" style="0"/>
+    <col min="9" max="9" width="16.42578125" customWidth="true" style="0"/>
+    <col min="10" max="10" width="1" customWidth="true" style="0"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="28.5">
+    <row r="1" spans="1:12" customHeight="1" ht="28.5">
       <c r="A1" s="23" t="s">
         <v>0</v>
       </c>
@@ -772,7 +751,7 @@
       <c r="K1" s="1"/>
       <c r="L1" s="1"/>
     </row>
-    <row r="2" spans="1:12" ht="33" customHeight="1">
+    <row r="2" spans="1:12" customHeight="1" ht="33">
       <c r="A2" s="31" t="s">
         <v>1</v>
       </c>
@@ -783,54 +762,54 @@
       </c>
       <c r="E2" s="13"/>
       <c r="F2" s="31" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G2" s="5"/>
       <c r="H2" s="3"/>
       <c r="I2" s="9" t="s">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="J2" s="8"/>
       <c r="K2" s="8"/>
     </row>
-    <row r="3" spans="1:12" ht="33.75" customHeight="1">
+    <row r="3" spans="1:12" customHeight="1" ht="33.75">
       <c r="A3" s="32" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="B3" s="22" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="C3" s="22"/>
       <c r="D3" s="22"/>
       <c r="E3" s="7"/>
       <c r="F3" s="35" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G3" s="5"/>
       <c r="H3" s="6" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="I3" s="4"/>
       <c r="J3" s="11"/>
     </row>
-    <row r="4" spans="1:12" ht="26.25" customHeight="1">
+    <row r="4" spans="1:12" customHeight="1" ht="26.25">
       <c r="A4" s="33" t="s">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="B4" s="34"/>
       <c r="C4" s="33" t="s">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D4" s="36"/>
       <c r="E4" s="34"/>
       <c r="F4" s="24" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="G4" s="25"/>
       <c r="H4" s="25"/>
       <c r="I4" s="26"/>
     </row>
-    <row r="5" spans="1:12" ht="35.25" customHeight="1">
+    <row r="5" spans="1:12" customHeight="1" ht="35.25">
       <c r="A5" s="17">
         <v>2100</v>
       </c>
@@ -847,7 +826,7 @@
       <c r="H5" s="15"/>
       <c r="I5" s="16"/>
     </row>
-    <row r="6" spans="1:12" ht="9" customHeight="1" thickBot="1">
+    <row r="6" spans="1:12" customHeight="1" ht="9">
       <c r="A6" s="10"/>
       <c r="B6" s="10"/>
       <c r="C6" s="10"/>
@@ -858,10 +837,10 @@
       <c r="H6" s="10"/>
       <c r="I6" s="10"/>
     </row>
-    <row r="7" spans="1:12" ht="12" customHeight="1">
+    <row r="7" spans="1:12" customHeight="1" ht="12">
       <c r="I7" s="2"/>
     </row>
-    <row r="8" spans="1:12" ht="32.1" customHeight="1">
+    <row r="8" spans="1:12" customHeight="1" ht="32.1">
       <c r="A8" s="39" t="s">
         <v>11</v>
       </c>
@@ -881,7 +860,7 @@
       <c r="I8" s="38"/>
       <c r="J8" s="11"/>
     </row>
-    <row r="9" spans="1:12" ht="32.1" customHeight="1">
+    <row r="9" spans="1:12" customHeight="1" ht="32.1">
       <c r="A9" s="27"/>
       <c r="B9" s="28"/>
       <c r="C9" s="27"/>
@@ -893,7 +872,7 @@
       <c r="I9" s="28"/>
       <c r="J9" s="11"/>
     </row>
-    <row r="10" spans="1:12" ht="32.1" customHeight="1">
+    <row r="10" spans="1:12" customHeight="1" ht="32.1">
       <c r="A10" s="29"/>
       <c r="B10" s="30"/>
       <c r="C10" s="29"/>
@@ -905,7 +884,7 @@
       <c r="I10" s="30"/>
       <c r="J10" s="11"/>
     </row>
-    <row r="11" spans="1:12" ht="32.1" customHeight="1">
+    <row r="11" spans="1:12" customHeight="1" ht="32.1">
       <c r="A11" s="27"/>
       <c r="B11" s="28"/>
       <c r="C11" s="27"/>
@@ -917,7 +896,7 @@
       <c r="I11" s="28"/>
       <c r="J11" s="11"/>
     </row>
-    <row r="12" spans="1:12" ht="32.1" customHeight="1">
+    <row r="12" spans="1:12" customHeight="1" ht="32.1">
       <c r="A12" s="29"/>
       <c r="B12" s="30"/>
       <c r="C12" s="29"/>
@@ -929,7 +908,7 @@
       <c r="I12" s="30"/>
       <c r="J12" s="11"/>
     </row>
-    <row r="13" spans="1:12" ht="32.1" customHeight="1">
+    <row r="13" spans="1:12" customHeight="1" ht="32.1">
       <c r="A13" s="27"/>
       <c r="B13" s="28"/>
       <c r="C13" s="27"/>
@@ -941,7 +920,7 @@
       <c r="I13" s="28"/>
       <c r="J13" s="11"/>
     </row>
-    <row r="14" spans="1:12" ht="32.1" customHeight="1">
+    <row r="14" spans="1:12" customHeight="1" ht="32.1">
       <c r="A14" s="29"/>
       <c r="B14" s="30"/>
       <c r="C14" s="29"/>
@@ -953,7 +932,7 @@
       <c r="I14" s="30"/>
       <c r="J14" s="11"/>
     </row>
-    <row r="15" spans="1:12" ht="32.1" customHeight="1">
+    <row r="15" spans="1:12" customHeight="1" ht="32.1">
       <c r="A15" s="27"/>
       <c r="B15" s="28"/>
       <c r="C15" s="27"/>
@@ -965,7 +944,7 @@
       <c r="I15" s="28"/>
       <c r="J15" s="11"/>
     </row>
-    <row r="16" spans="1:12" ht="32.1" customHeight="1">
+    <row r="16" spans="1:12" customHeight="1" ht="32.1">
       <c r="A16" s="29"/>
       <c r="B16" s="30"/>
       <c r="C16" s="29"/>
@@ -977,7 +956,7 @@
       <c r="I16" s="30"/>
       <c r="J16" s="11"/>
     </row>
-    <row r="17" spans="1:10" ht="32.1" customHeight="1">
+    <row r="17" spans="1:12" customHeight="1" ht="32.1">
       <c r="A17" s="27"/>
       <c r="B17" s="28"/>
       <c r="C17" s="27"/>
@@ -989,7 +968,7 @@
       <c r="I17" s="28"/>
       <c r="J17" s="11"/>
     </row>
-    <row r="18" spans="1:10" ht="32.1" customHeight="1">
+    <row r="18" spans="1:12" customHeight="1" ht="32.1">
       <c r="A18" s="29"/>
       <c r="B18" s="30"/>
       <c r="C18" s="29"/>
@@ -1001,7 +980,7 @@
       <c r="I18" s="30"/>
       <c r="J18" s="11"/>
     </row>
-    <row r="19" spans="1:10" ht="32.1" customHeight="1">
+    <row r="19" spans="1:12" customHeight="1" ht="32.1">
       <c r="A19" s="27"/>
       <c r="B19" s="28"/>
       <c r="C19" s="27"/>
@@ -1013,7 +992,7 @@
       <c r="I19" s="28"/>
       <c r="J19" s="11"/>
     </row>
-    <row r="20" spans="1:10" ht="32.1" customHeight="1">
+    <row r="20" spans="1:12" customHeight="1" ht="32.1">
       <c r="A20" s="29"/>
       <c r="B20" s="30"/>
       <c r="C20" s="29"/>
@@ -1025,7 +1004,7 @@
       <c r="I20" s="30"/>
       <c r="J20" s="11"/>
     </row>
-    <row r="21" spans="1:10" ht="32.1" customHeight="1">
+    <row r="21" spans="1:12" customHeight="1" ht="32.1">
       <c r="A21" s="27"/>
       <c r="B21" s="28"/>
       <c r="C21" s="27"/>
@@ -1037,7 +1016,7 @@
       <c r="I21" s="28"/>
       <c r="J21" s="11"/>
     </row>
-    <row r="22" spans="1:10" ht="32.1" customHeight="1">
+    <row r="22" spans="1:12" customHeight="1" ht="32.1">
       <c r="A22" s="29"/>
       <c r="B22" s="30"/>
       <c r="C22" s="29"/>
@@ -1049,7 +1028,7 @@
       <c r="I22" s="30"/>
       <c r="J22" s="11"/>
     </row>
-    <row r="23" spans="1:10" ht="32.1" customHeight="1">
+    <row r="23" spans="1:12" customHeight="1" ht="32.1">
       <c r="A23" s="27"/>
       <c r="B23" s="28"/>
       <c r="C23" s="27"/>
@@ -1061,7 +1040,7 @@
       <c r="I23" s="28"/>
       <c r="J23" s="11"/>
     </row>
-    <row r="24" spans="1:10" ht="32.1" customHeight="1">
+    <row r="24" spans="1:12" customHeight="1" ht="32.1">
       <c r="A24" s="29"/>
       <c r="B24" s="30"/>
       <c r="C24" s="29"/>
@@ -1073,7 +1052,7 @@
       <c r="I24" s="30"/>
       <c r="J24" s="11"/>
     </row>
-    <row r="25" spans="1:10" ht="32.1" customHeight="1">
+    <row r="25" spans="1:12" customHeight="1" ht="32.1">
       <c r="A25" s="27"/>
       <c r="B25" s="28"/>
       <c r="C25" s="27"/>
@@ -1085,7 +1064,7 @@
       <c r="I25" s="28"/>
       <c r="J25" s="11"/>
     </row>
-    <row r="26" spans="1:10" ht="32.1" customHeight="1">
+    <row r="26" spans="1:12" customHeight="1" ht="32.1">
       <c r="A26" s="37" t="s">
         <v>11</v>
       </c>
@@ -1105,7 +1084,7 @@
       <c r="I26" s="38"/>
       <c r="J26" s="11"/>
     </row>
-    <row r="27" spans="1:10" ht="32.1" customHeight="1">
+    <row r="27" spans="1:12" customHeight="1" ht="32.1">
       <c r="A27" s="27"/>
       <c r="B27" s="28"/>
       <c r="C27" s="27"/>
@@ -1117,7 +1096,7 @@
       <c r="I27" s="28"/>
       <c r="J27" s="11"/>
     </row>
-    <row r="28" spans="1:10" ht="32.1" customHeight="1">
+    <row r="28" spans="1:12" customHeight="1" ht="32.1">
       <c r="A28" s="29"/>
       <c r="B28" s="30"/>
       <c r="C28" s="29"/>
@@ -1129,7 +1108,7 @@
       <c r="I28" s="30"/>
       <c r="J28" s="11"/>
     </row>
-    <row r="29" spans="1:10" ht="32.1" customHeight="1">
+    <row r="29" spans="1:12" customHeight="1" ht="32.1">
       <c r="A29" s="27"/>
       <c r="B29" s="28"/>
       <c r="C29" s="27"/>
@@ -1141,7 +1120,7 @@
       <c r="I29" s="28"/>
       <c r="J29" s="11"/>
     </row>
-    <row r="30" spans="1:10" ht="32.1" customHeight="1">
+    <row r="30" spans="1:12" customHeight="1" ht="32.1">
       <c r="A30" s="29"/>
       <c r="B30" s="30"/>
       <c r="C30" s="29"/>
@@ -1153,7 +1132,7 @@
       <c r="I30" s="30"/>
       <c r="J30" s="11"/>
     </row>
-    <row r="31" spans="1:10" ht="32.1" customHeight="1">
+    <row r="31" spans="1:12" customHeight="1" ht="32.1">
       <c r="A31" s="27"/>
       <c r="B31" s="28"/>
       <c r="C31" s="27"/>
@@ -1165,7 +1144,7 @@
       <c r="I31" s="28"/>
       <c r="J31" s="11"/>
     </row>
-    <row r="32" spans="1:10" ht="32.1" customHeight="1">
+    <row r="32" spans="1:12" customHeight="1" ht="32.1">
       <c r="A32" s="29"/>
       <c r="B32" s="30"/>
       <c r="C32" s="29"/>
@@ -1177,7 +1156,7 @@
       <c r="I32" s="30"/>
       <c r="J32" s="11"/>
     </row>
-    <row r="33" spans="1:10" ht="32.1" customHeight="1">
+    <row r="33" spans="1:12" customHeight="1" ht="32.1">
       <c r="A33" s="27"/>
       <c r="B33" s="28"/>
       <c r="C33" s="27"/>
@@ -1189,7 +1168,7 @@
       <c r="I33" s="28"/>
       <c r="J33" s="11"/>
     </row>
-    <row r="34" spans="1:10" ht="32.1" customHeight="1">
+    <row r="34" spans="1:12" customHeight="1" ht="32.1">
       <c r="A34" s="29"/>
       <c r="B34" s="30"/>
       <c r="C34" s="29"/>
@@ -1201,7 +1180,7 @@
       <c r="I34" s="30"/>
       <c r="J34" s="11"/>
     </row>
-    <row r="35" spans="1:10" ht="32.1" customHeight="1">
+    <row r="35" spans="1:12" customHeight="1" ht="32.1">
       <c r="A35" s="27"/>
       <c r="B35" s="28"/>
       <c r="C35" s="27"/>
@@ -1213,7 +1192,7 @@
       <c r="I35" s="28"/>
       <c r="J35" s="11"/>
     </row>
-    <row r="36" spans="1:10" ht="32.1" customHeight="1">
+    <row r="36" spans="1:12" customHeight="1" ht="32.1">
       <c r="A36" s="29"/>
       <c r="B36" s="30"/>
       <c r="C36" s="29"/>
@@ -1225,7 +1204,7 @@
       <c r="I36" s="30"/>
       <c r="J36" s="11"/>
     </row>
-    <row r="37" spans="1:10" ht="32.1" customHeight="1">
+    <row r="37" spans="1:12" customHeight="1" ht="32.1">
       <c r="A37" s="27"/>
       <c r="B37" s="28"/>
       <c r="C37" s="27"/>
@@ -1237,7 +1216,7 @@
       <c r="I37" s="28"/>
       <c r="J37" s="11"/>
     </row>
-    <row r="38" spans="1:10" ht="32.1" customHeight="1">
+    <row r="38" spans="1:12" customHeight="1" ht="32.1">
       <c r="A38" s="29"/>
       <c r="B38" s="30"/>
       <c r="C38" s="29"/>
@@ -1249,7 +1228,7 @@
       <c r="I38" s="30"/>
       <c r="J38" s="11"/>
     </row>
-    <row r="39" spans="1:10" ht="32.1" customHeight="1">
+    <row r="39" spans="1:12" customHeight="1" ht="32.1">
       <c r="A39" s="27"/>
       <c r="B39" s="28"/>
       <c r="C39" s="27"/>
@@ -1261,7 +1240,7 @@
       <c r="I39" s="28"/>
       <c r="J39" s="11"/>
     </row>
-    <row r="40" spans="1:10" ht="32.1" customHeight="1">
+    <row r="40" spans="1:12" customHeight="1" ht="32.1">
       <c r="A40" s="29"/>
       <c r="B40" s="30"/>
       <c r="C40" s="29"/>
@@ -1273,7 +1252,7 @@
       <c r="I40" s="30"/>
       <c r="J40" s="11"/>
     </row>
-    <row r="41" spans="1:10" ht="32.1" customHeight="1">
+    <row r="41" spans="1:12" customHeight="1" ht="32.1">
       <c r="A41" s="27"/>
       <c r="B41" s="28"/>
       <c r="C41" s="27"/>
@@ -1285,7 +1264,7 @@
       <c r="I41" s="28"/>
       <c r="J41" s="11"/>
     </row>
-    <row r="42" spans="1:10" ht="32.1" customHeight="1">
+    <row r="42" spans="1:12" customHeight="1" ht="32.1">
       <c r="A42" s="29"/>
       <c r="B42" s="30"/>
       <c r="C42" s="29"/>
@@ -1297,7 +1276,7 @@
       <c r="I42" s="30"/>
       <c r="J42" s="11"/>
     </row>
-    <row r="43" spans="1:10" ht="32.1" customHeight="1">
+    <row r="43" spans="1:12" customHeight="1" ht="32.1">
       <c r="A43" s="27"/>
       <c r="B43" s="28"/>
       <c r="C43" s="27"/>
@@ -1309,7 +1288,7 @@
       <c r="I43" s="28"/>
       <c r="J43" s="11"/>
     </row>
-    <row r="44" spans="1:10" ht="32.1" customHeight="1">
+    <row r="44" spans="1:12" customHeight="1" ht="32.1">
       <c r="A44" s="29"/>
       <c r="B44" s="30"/>
       <c r="C44" s="29"/>
@@ -1321,7 +1300,7 @@
       <c r="I44" s="30"/>
       <c r="J44" s="11"/>
     </row>
-    <row r="45" spans="1:10" ht="32.1" customHeight="1">
+    <row r="45" spans="1:12" customHeight="1" ht="32.1">
       <c r="A45" s="27"/>
       <c r="B45" s="28"/>
       <c r="C45" s="27"/>
@@ -1333,7 +1312,7 @@
       <c r="I45" s="28"/>
       <c r="J45" s="11"/>
     </row>
-    <row r="46" spans="1:10" ht="32.1" customHeight="1">
+    <row r="46" spans="1:12" customHeight="1" ht="32.1">
       <c r="A46" s="29"/>
       <c r="B46" s="30"/>
       <c r="C46" s="29"/>
@@ -1345,7 +1324,7 @@
       <c r="I46" s="30"/>
       <c r="J46" s="11"/>
     </row>
-    <row r="47" spans="1:10" ht="32.1" customHeight="1">
+    <row r="47" spans="1:12" customHeight="1" ht="32.1">
       <c r="A47" s="27"/>
       <c r="B47" s="28"/>
       <c r="C47" s="27"/>
@@ -1357,7 +1336,7 @@
       <c r="I47" s="28"/>
       <c r="J47" s="11"/>
     </row>
-    <row r="48" spans="1:10" ht="32.1" customHeight="1">
+    <row r="48" spans="1:12" customHeight="1" ht="32.1">
       <c r="A48" s="29"/>
       <c r="B48" s="30"/>
       <c r="C48" s="29"/>
@@ -1370,7 +1349,7 @@
       <c r="J48" s="11"/>
     </row>
   </sheetData>
-  <mergeCells count="173">
+  <mergeCells>
     <mergeCell ref="A48:B48"/>
     <mergeCell ref="C48:D48"/>
     <mergeCell ref="E48:G48"/>
@@ -1545,25 +1524,837 @@
     <mergeCell ref="C5:E5"/>
     <mergeCell ref="B3:D3"/>
   </mergeCells>
-  <pageMargins left="0.70866141732283472" right="0.51181102362204722" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <printOptions gridLines="false" gridLinesSet="true"/>
+  <pageMargins left="0.70866141732283" right="0.51181102362205" top="0.74803149606299" bottom="0.74803149606299" header="0.31496062992126" footer="0.31496062992126"/>
+  <pageSetup paperSize="9" orientation="portrait" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" r:id="rId1ps"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xml:space="preserve" mc:Ignorable="x14ac">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+  </sheetPr>
+  <dimension ref="A1:L48"/>
+  <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetData>
+    <row r="1" spans="1:12">
+      <c r="A1" s="23" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="23"/>
+      <c r="C1" s="23"/>
+      <c r="D1" s="23"/>
+      <c r="E1" s="23"/>
+      <c r="F1" s="23"/>
+      <c r="G1" s="23"/>
+      <c r="H1" s="23"/>
+      <c r="I1" s="23"/>
+      <c r="J1" s="1"/>
+      <c r="K1" s="1"/>
+      <c r="L1" s="1"/>
+    </row>
+    <row r="2" spans="1:12">
+      <c r="A2" s="31" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="12">
+        <v>46167</v>
+      </c>
+      <c r="E2" s="13"/>
+      <c r="F2" s="31" t="s">
+        <v>2</v>
+      </c>
+      <c r="G2" s="5"/>
+      <c r="H2" s="3"/>
+      <c r="I2" s="9" t="s">
+        <v>3</v>
+      </c>
+      <c r="J2" s="8"/>
+      <c r="K2" s="8"/>
+    </row>
+    <row r="3" spans="1:12">
+      <c r="A3" s="32" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="C3" s="7"/>
+      <c r="D3" s="7"/>
+      <c r="E3" s="7"/>
+      <c r="F3" s="35" t="s">
+        <v>6</v>
+      </c>
+      <c r="G3" s="5"/>
+      <c r="H3" s="6" t="inlineStr">
+        <is>
+          <r>
+            <t xml:space="preserve">MLT  DROP  </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="false"/>
+              <i val="false"/>
+              <strike val="false"/>
+              <color rgb="FF000000"/>
+              <sz val="11"/>
+              <u val="single"/>
+            </rPr>
+            <t xml:space="preserve">BLOWN</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="false"/>
+              <i val="false"/>
+              <strike val="false"/>
+              <color rgb="FF000000"/>
+              <sz val="11"/>
+              <u val="none"/>
+            </rPr>
+            <t xml:space="preserve">  FLAT</t>
+          </r>
+        </is>
+      </c>
+      <c r="I3" s="4"/>
+      <c r="J3" s="11"/>
+    </row>
+    <row r="4" spans="1:12">
+      <c r="A4" s="33" t="s">
+        <v>8</v>
+      </c>
+      <c r="B4" s="34"/>
+      <c r="C4" s="33" t="s">
+        <v>9</v>
+      </c>
+      <c r="D4" s="36"/>
+      <c r="E4" s="34"/>
+      <c r="F4" s="24" t="s">
+        <v>10</v>
+      </c>
+      <c r="G4" s="25"/>
+      <c r="H4" s="25"/>
+      <c r="I4" s="26"/>
+    </row>
+    <row r="5" spans="1:12">
+      <c r="A5" s="17">
+        <v>2100</v>
+      </c>
+      <c r="B5" s="18"/>
+      <c r="C5" s="19">
+        <v>4500</v>
+      </c>
+      <c r="D5" s="20"/>
+      <c r="E5" s="21"/>
+      <c r="F5" s="14">
+        <v>2</v>
+      </c>
+      <c r="G5" s="15"/>
+      <c r="H5" s="15"/>
+      <c r="I5" s="16"/>
+    </row>
+    <row r="6" spans="1:12">
+      <c r="A6" s="10"/>
+      <c r="B6" s="10"/>
+      <c r="C6" s="10"/>
+      <c r="D6" s="10"/>
+      <c r="E6" s="10"/>
+      <c r="F6" s="10"/>
+      <c r="G6" s="10"/>
+      <c r="H6" s="10"/>
+      <c r="I6" s="10"/>
+    </row>
+    <row r="7" spans="1:12"/>
+    <row r="8" spans="1:12">
+      <c r="A8" s="37" t="s">
+        <v>11</v>
+      </c>
+      <c r="B8" s="38"/>
+      <c r="C8" s="37" t="s">
+        <v>12</v>
+      </c>
+      <c r="D8" s="38"/>
+      <c r="E8" s="37" t="s">
+        <v>13</v>
+      </c>
+      <c r="F8" s="38"/>
+      <c r="G8" s="38"/>
+      <c r="H8" s="37" t="s">
+        <v>14</v>
+      </c>
+      <c r="I8" s="38"/>
+      <c r="J8" s="11"/>
+    </row>
+    <row r="9" spans="1:12">
+      <c r="A9" s="27"/>
+      <c r="B9" s="28"/>
+      <c r="C9" s="27"/>
+      <c r="D9" s="28"/>
+      <c r="E9" s="27"/>
+      <c r="F9" s="28"/>
+      <c r="G9" s="28"/>
+      <c r="H9" s="27"/>
+      <c r="I9" s="28"/>
+      <c r="J9" s="11"/>
+    </row>
+    <row r="10" spans="1:12">
+      <c r="A10" s="29"/>
+      <c r="B10" s="30"/>
+      <c r="C10" s="29"/>
+      <c r="D10" s="30"/>
+      <c r="E10" s="29"/>
+      <c r="F10" s="30"/>
+      <c r="G10" s="30"/>
+      <c r="H10" s="29"/>
+      <c r="I10" s="30"/>
+      <c r="J10" s="11"/>
+    </row>
+    <row r="11" spans="1:12">
+      <c r="A11" s="27"/>
+      <c r="B11" s="28"/>
+      <c r="C11" s="27"/>
+      <c r="D11" s="28"/>
+      <c r="E11" s="27"/>
+      <c r="F11" s="28"/>
+      <c r="G11" s="28"/>
+      <c r="H11" s="27"/>
+      <c r="I11" s="28"/>
+      <c r="J11" s="11"/>
+    </row>
+    <row r="12" spans="1:12">
+      <c r="A12" s="29"/>
+      <c r="B12" s="30"/>
+      <c r="C12" s="29"/>
+      <c r="D12" s="30"/>
+      <c r="E12" s="29"/>
+      <c r="F12" s="30"/>
+      <c r="G12" s="30"/>
+      <c r="H12" s="29"/>
+      <c r="I12" s="30"/>
+      <c r="J12" s="11"/>
+    </row>
+    <row r="13" spans="1:12">
+      <c r="A13" s="27"/>
+      <c r="B13" s="28"/>
+      <c r="C13" s="27"/>
+      <c r="D13" s="28"/>
+      <c r="E13" s="27"/>
+      <c r="F13" s="28"/>
+      <c r="G13" s="28"/>
+      <c r="H13" s="27"/>
+      <c r="I13" s="28"/>
+      <c r="J13" s="11"/>
+    </row>
+    <row r="14" spans="1:12">
+      <c r="A14" s="29"/>
+      <c r="B14" s="30"/>
+      <c r="C14" s="29"/>
+      <c r="D14" s="30"/>
+      <c r="E14" s="29"/>
+      <c r="F14" s="30"/>
+      <c r="G14" s="30"/>
+      <c r="H14" s="29"/>
+      <c r="I14" s="30"/>
+      <c r="J14" s="11"/>
+    </row>
+    <row r="15" spans="1:12">
+      <c r="A15" s="27"/>
+      <c r="B15" s="28"/>
+      <c r="C15" s="27"/>
+      <c r="D15" s="28"/>
+      <c r="E15" s="27"/>
+      <c r="F15" s="28"/>
+      <c r="G15" s="28"/>
+      <c r="H15" s="27"/>
+      <c r="I15" s="28"/>
+      <c r="J15" s="11"/>
+    </row>
+    <row r="16" spans="1:12">
+      <c r="A16" s="29"/>
+      <c r="B16" s="30"/>
+      <c r="C16" s="29"/>
+      <c r="D16" s="30"/>
+      <c r="E16" s="29"/>
+      <c r="F16" s="30"/>
+      <c r="G16" s="30"/>
+      <c r="H16" s="29"/>
+      <c r="I16" s="30"/>
+      <c r="J16" s="11"/>
+    </row>
+    <row r="17" spans="1:12">
+      <c r="A17" s="27"/>
+      <c r="B17" s="28"/>
+      <c r="C17" s="27"/>
+      <c r="D17" s="28"/>
+      <c r="E17" s="27"/>
+      <c r="F17" s="28"/>
+      <c r="G17" s="28"/>
+      <c r="H17" s="27"/>
+      <c r="I17" s="28"/>
+      <c r="J17" s="11"/>
+    </row>
+    <row r="18" spans="1:12">
+      <c r="A18" s="29"/>
+      <c r="B18" s="30"/>
+      <c r="C18" s="29"/>
+      <c r="D18" s="30"/>
+      <c r="E18" s="29"/>
+      <c r="F18" s="30"/>
+      <c r="G18" s="30"/>
+      <c r="H18" s="29"/>
+      <c r="I18" s="30"/>
+      <c r="J18" s="11"/>
+    </row>
+    <row r="19" spans="1:12">
+      <c r="A19" s="27"/>
+      <c r="B19" s="28"/>
+      <c r="C19" s="27"/>
+      <c r="D19" s="28"/>
+      <c r="E19" s="27"/>
+      <c r="F19" s="28"/>
+      <c r="G19" s="28"/>
+      <c r="H19" s="27"/>
+      <c r="I19" s="28"/>
+      <c r="J19" s="11"/>
+    </row>
+    <row r="20" spans="1:12">
+      <c r="A20" s="29"/>
+      <c r="B20" s="30"/>
+      <c r="C20" s="29"/>
+      <c r="D20" s="30"/>
+      <c r="E20" s="29"/>
+      <c r="F20" s="30"/>
+      <c r="G20" s="30"/>
+      <c r="H20" s="29"/>
+      <c r="I20" s="30"/>
+      <c r="J20" s="11"/>
+    </row>
+    <row r="21" spans="1:12">
+      <c r="A21" s="27"/>
+      <c r="B21" s="28"/>
+      <c r="C21" s="27"/>
+      <c r="D21" s="28"/>
+      <c r="E21" s="27"/>
+      <c r="F21" s="28"/>
+      <c r="G21" s="28"/>
+      <c r="H21" s="27"/>
+      <c r="I21" s="28"/>
+      <c r="J21" s="11"/>
+    </row>
+    <row r="22" spans="1:12">
+      <c r="A22" s="29"/>
+      <c r="B22" s="30"/>
+      <c r="C22" s="29"/>
+      <c r="D22" s="30"/>
+      <c r="E22" s="29"/>
+      <c r="F22" s="30"/>
+      <c r="G22" s="30"/>
+      <c r="H22" s="29"/>
+      <c r="I22" s="30"/>
+      <c r="J22" s="11"/>
+    </row>
+    <row r="23" spans="1:12">
+      <c r="A23" s="27"/>
+      <c r="B23" s="28"/>
+      <c r="C23" s="27"/>
+      <c r="D23" s="28"/>
+      <c r="E23" s="27"/>
+      <c r="F23" s="28"/>
+      <c r="G23" s="28"/>
+      <c r="H23" s="27"/>
+      <c r="I23" s="28"/>
+      <c r="J23" s="11"/>
+    </row>
+    <row r="24" spans="1:12">
+      <c r="A24" s="29"/>
+      <c r="B24" s="30"/>
+      <c r="C24" s="29"/>
+      <c r="D24" s="30"/>
+      <c r="E24" s="29"/>
+      <c r="F24" s="30"/>
+      <c r="G24" s="30"/>
+      <c r="H24" s="29"/>
+      <c r="I24" s="30"/>
+      <c r="J24" s="11"/>
+    </row>
+    <row r="25" spans="1:12">
+      <c r="A25" s="27"/>
+      <c r="B25" s="28"/>
+      <c r="C25" s="27"/>
+      <c r="D25" s="28"/>
+      <c r="E25" s="27"/>
+      <c r="F25" s="28"/>
+      <c r="G25" s="28"/>
+      <c r="H25" s="27"/>
+      <c r="I25" s="28"/>
+      <c r="J25" s="11"/>
+    </row>
+    <row r="26" spans="1:12">
+      <c r="A26" s="37" t="s">
+        <v>11</v>
+      </c>
+      <c r="B26" s="38"/>
+      <c r="C26" s="37" t="s">
+        <v>12</v>
+      </c>
+      <c r="D26" s="38"/>
+      <c r="E26" s="37" t="s">
+        <v>13</v>
+      </c>
+      <c r="F26" s="38"/>
+      <c r="G26" s="38"/>
+      <c r="H26" s="37" t="s">
+        <v>14</v>
+      </c>
+      <c r="I26" s="38"/>
+      <c r="J26" s="11"/>
+    </row>
+    <row r="27" spans="1:12">
+      <c r="A27" s="27"/>
+      <c r="B27" s="28"/>
+      <c r="C27" s="27"/>
+      <c r="D27" s="28"/>
+      <c r="E27" s="27"/>
+      <c r="F27" s="28"/>
+      <c r="G27" s="28"/>
+      <c r="H27" s="27"/>
+      <c r="I27" s="28"/>
+      <c r="J27" s="11"/>
+    </row>
+    <row r="28" spans="1:12">
+      <c r="A28" s="29"/>
+      <c r="B28" s="30"/>
+      <c r="C28" s="29"/>
+      <c r="D28" s="30"/>
+      <c r="E28" s="29"/>
+      <c r="F28" s="30"/>
+      <c r="G28" s="30"/>
+      <c r="H28" s="29"/>
+      <c r="I28" s="30"/>
+      <c r="J28" s="11"/>
+    </row>
+    <row r="29" spans="1:12">
+      <c r="A29" s="27"/>
+      <c r="B29" s="28"/>
+      <c r="C29" s="27"/>
+      <c r="D29" s="28"/>
+      <c r="E29" s="27"/>
+      <c r="F29" s="28"/>
+      <c r="G29" s="28"/>
+      <c r="H29" s="27"/>
+      <c r="I29" s="28"/>
+      <c r="J29" s="11"/>
+    </row>
+    <row r="30" spans="1:12">
+      <c r="A30" s="29"/>
+      <c r="B30" s="30"/>
+      <c r="C30" s="29"/>
+      <c r="D30" s="30"/>
+      <c r="E30" s="29"/>
+      <c r="F30" s="30"/>
+      <c r="G30" s="30"/>
+      <c r="H30" s="29"/>
+      <c r="I30" s="30"/>
+      <c r="J30" s="11"/>
+    </row>
+    <row r="31" spans="1:12">
+      <c r="A31" s="27"/>
+      <c r="B31" s="28"/>
+      <c r="C31" s="27"/>
+      <c r="D31" s="28"/>
+      <c r="E31" s="27"/>
+      <c r="F31" s="28"/>
+      <c r="G31" s="28"/>
+      <c r="H31" s="27"/>
+      <c r="I31" s="28"/>
+      <c r="J31" s="11"/>
+    </row>
+    <row r="32" spans="1:12">
+      <c r="A32" s="29"/>
+      <c r="B32" s="30"/>
+      <c r="C32" s="29"/>
+      <c r="D32" s="30"/>
+      <c r="E32" s="29"/>
+      <c r="F32" s="30"/>
+      <c r="G32" s="30"/>
+      <c r="H32" s="29"/>
+      <c r="I32" s="30"/>
+      <c r="J32" s="11"/>
+    </row>
+    <row r="33" spans="1:12">
+      <c r="A33" s="27"/>
+      <c r="B33" s="28"/>
+      <c r="C33" s="27"/>
+      <c r="D33" s="28"/>
+      <c r="E33" s="27"/>
+      <c r="F33" s="28"/>
+      <c r="G33" s="28"/>
+      <c r="H33" s="27"/>
+      <c r="I33" s="28"/>
+      <c r="J33" s="11"/>
+    </row>
+    <row r="34" spans="1:12">
+      <c r="A34" s="29"/>
+      <c r="B34" s="30"/>
+      <c r="C34" s="29"/>
+      <c r="D34" s="30"/>
+      <c r="E34" s="29"/>
+      <c r="F34" s="30"/>
+      <c r="G34" s="30"/>
+      <c r="H34" s="29"/>
+      <c r="I34" s="30"/>
+      <c r="J34" s="11"/>
+    </row>
+    <row r="35" spans="1:12">
+      <c r="A35" s="27"/>
+      <c r="B35" s="28"/>
+      <c r="C35" s="27"/>
+      <c r="D35" s="28"/>
+      <c r="E35" s="27"/>
+      <c r="F35" s="28"/>
+      <c r="G35" s="28"/>
+      <c r="H35" s="27"/>
+      <c r="I35" s="28"/>
+      <c r="J35" s="11"/>
+    </row>
+    <row r="36" spans="1:12">
+      <c r="A36" s="29"/>
+      <c r="B36" s="30"/>
+      <c r="C36" s="29"/>
+      <c r="D36" s="30"/>
+      <c r="E36" s="29"/>
+      <c r="F36" s="30"/>
+      <c r="G36" s="30"/>
+      <c r="H36" s="29"/>
+      <c r="I36" s="30"/>
+      <c r="J36" s="11"/>
+    </row>
+    <row r="37" spans="1:12">
+      <c r="A37" s="27"/>
+      <c r="B37" s="28"/>
+      <c r="C37" s="27"/>
+      <c r="D37" s="28"/>
+      <c r="E37" s="27"/>
+      <c r="F37" s="28"/>
+      <c r="G37" s="28"/>
+      <c r="H37" s="27"/>
+      <c r="I37" s="28"/>
+      <c r="J37" s="11"/>
+    </row>
+    <row r="38" spans="1:12">
+      <c r="A38" s="29"/>
+      <c r="B38" s="30"/>
+      <c r="C38" s="29"/>
+      <c r="D38" s="30"/>
+      <c r="E38" s="29"/>
+      <c r="F38" s="30"/>
+      <c r="G38" s="30"/>
+      <c r="H38" s="29"/>
+      <c r="I38" s="30"/>
+      <c r="J38" s="11"/>
+    </row>
+    <row r="39" spans="1:12">
+      <c r="A39" s="27"/>
+      <c r="B39" s="28"/>
+      <c r="C39" s="27"/>
+      <c r="D39" s="28"/>
+      <c r="E39" s="27"/>
+      <c r="F39" s="28"/>
+      <c r="G39" s="28"/>
+      <c r="H39" s="27"/>
+      <c r="I39" s="28"/>
+      <c r="J39" s="11"/>
+    </row>
+    <row r="40" spans="1:12">
+      <c r="A40" s="29"/>
+      <c r="B40" s="30"/>
+      <c r="C40" s="29"/>
+      <c r="D40" s="30"/>
+      <c r="E40" s="29"/>
+      <c r="F40" s="30"/>
+      <c r="G40" s="30"/>
+      <c r="H40" s="29"/>
+      <c r="I40" s="30"/>
+      <c r="J40" s="11"/>
+    </row>
+    <row r="41" spans="1:12">
+      <c r="A41" s="27"/>
+      <c r="B41" s="28"/>
+      <c r="C41" s="27"/>
+      <c r="D41" s="28"/>
+      <c r="E41" s="27"/>
+      <c r="F41" s="28"/>
+      <c r="G41" s="28"/>
+      <c r="H41" s="27"/>
+      <c r="I41" s="28"/>
+      <c r="J41" s="11"/>
+    </row>
+    <row r="42" spans="1:12">
+      <c r="A42" s="29"/>
+      <c r="B42" s="30"/>
+      <c r="C42" s="29"/>
+      <c r="D42" s="30"/>
+      <c r="E42" s="29"/>
+      <c r="F42" s="30"/>
+      <c r="G42" s="30"/>
+      <c r="H42" s="29"/>
+      <c r="I42" s="30"/>
+      <c r="J42" s="11"/>
+    </row>
+    <row r="43" spans="1:12">
+      <c r="A43" s="27"/>
+      <c r="B43" s="28"/>
+      <c r="C43" s="27"/>
+      <c r="D43" s="28"/>
+      <c r="E43" s="27"/>
+      <c r="F43" s="28"/>
+      <c r="G43" s="28"/>
+      <c r="H43" s="27"/>
+      <c r="I43" s="28"/>
+      <c r="J43" s="11"/>
+    </row>
+    <row r="44" spans="1:12">
+      <c r="A44" s="29"/>
+      <c r="B44" s="30"/>
+      <c r="C44" s="29"/>
+      <c r="D44" s="30"/>
+      <c r="E44" s="29"/>
+      <c r="F44" s="30"/>
+      <c r="G44" s="30"/>
+      <c r="H44" s="29"/>
+      <c r="I44" s="30"/>
+      <c r="J44" s="11"/>
+    </row>
+    <row r="45" spans="1:12">
+      <c r="A45" s="27"/>
+      <c r="B45" s="28"/>
+      <c r="C45" s="27"/>
+      <c r="D45" s="28"/>
+      <c r="E45" s="27"/>
+      <c r="F45" s="28"/>
+      <c r="G45" s="28"/>
+      <c r="H45" s="27"/>
+      <c r="I45" s="28"/>
+      <c r="J45" s="11"/>
+    </row>
+    <row r="46" spans="1:12">
+      <c r="A46" s="29"/>
+      <c r="B46" s="30"/>
+      <c r="C46" s="29"/>
+      <c r="D46" s="30"/>
+      <c r="E46" s="29"/>
+      <c r="F46" s="30"/>
+      <c r="G46" s="30"/>
+      <c r="H46" s="29"/>
+      <c r="I46" s="30"/>
+      <c r="J46" s="11"/>
+    </row>
+    <row r="47" spans="1:12">
+      <c r="A47" s="27"/>
+      <c r="B47" s="28"/>
+      <c r="C47" s="27"/>
+      <c r="D47" s="28"/>
+      <c r="E47" s="27"/>
+      <c r="F47" s="28"/>
+      <c r="G47" s="28"/>
+      <c r="H47" s="27"/>
+      <c r="I47" s="28"/>
+      <c r="J47" s="11"/>
+    </row>
+    <row r="48" spans="1:12">
+      <c r="A48" s="29"/>
+      <c r="B48" s="30"/>
+      <c r="C48" s="29"/>
+      <c r="D48" s="30"/>
+      <c r="E48" s="29"/>
+      <c r="F48" s="30"/>
+      <c r="G48" s="30"/>
+      <c r="H48" s="29"/>
+      <c r="I48" s="30"/>
+      <c r="J48" s="11"/>
+    </row>
+  </sheetData>
+  <mergeCells>
+    <mergeCell ref="A48:B48"/>
+    <mergeCell ref="C48:D48"/>
+    <mergeCell ref="E48:G48"/>
+    <mergeCell ref="H48:I48"/>
+    <mergeCell ref="A46:B46"/>
+    <mergeCell ref="C46:D46"/>
+    <mergeCell ref="E46:G46"/>
+    <mergeCell ref="H46:I46"/>
+    <mergeCell ref="A47:B47"/>
+    <mergeCell ref="C47:D47"/>
+    <mergeCell ref="E47:G47"/>
+    <mergeCell ref="H47:I47"/>
+    <mergeCell ref="A44:B44"/>
+    <mergeCell ref="C44:D44"/>
+    <mergeCell ref="E44:G44"/>
+    <mergeCell ref="H44:I44"/>
+    <mergeCell ref="A45:B45"/>
+    <mergeCell ref="C45:D45"/>
+    <mergeCell ref="E45:G45"/>
+    <mergeCell ref="H45:I45"/>
+    <mergeCell ref="A42:B42"/>
+    <mergeCell ref="C42:D42"/>
+    <mergeCell ref="E42:G42"/>
+    <mergeCell ref="H42:I42"/>
+    <mergeCell ref="A43:B43"/>
+    <mergeCell ref="C43:D43"/>
+    <mergeCell ref="E43:G43"/>
+    <mergeCell ref="H43:I43"/>
+    <mergeCell ref="A40:B40"/>
+    <mergeCell ref="C40:D40"/>
+    <mergeCell ref="E40:G40"/>
+    <mergeCell ref="H40:I40"/>
+    <mergeCell ref="A41:B41"/>
+    <mergeCell ref="C41:D41"/>
+    <mergeCell ref="E41:G41"/>
+    <mergeCell ref="H41:I41"/>
+    <mergeCell ref="A38:B38"/>
+    <mergeCell ref="C38:D38"/>
+    <mergeCell ref="E38:G38"/>
+    <mergeCell ref="H38:I38"/>
+    <mergeCell ref="A39:B39"/>
+    <mergeCell ref="C39:D39"/>
+    <mergeCell ref="E39:G39"/>
+    <mergeCell ref="H39:I39"/>
+    <mergeCell ref="A36:B36"/>
+    <mergeCell ref="C36:D36"/>
+    <mergeCell ref="E36:G36"/>
+    <mergeCell ref="H36:I36"/>
+    <mergeCell ref="A37:B37"/>
+    <mergeCell ref="C37:D37"/>
+    <mergeCell ref="E37:G37"/>
+    <mergeCell ref="H37:I37"/>
+    <mergeCell ref="A34:B34"/>
+    <mergeCell ref="C34:D34"/>
+    <mergeCell ref="E34:G34"/>
+    <mergeCell ref="H34:I34"/>
+    <mergeCell ref="A35:B35"/>
+    <mergeCell ref="C35:D35"/>
+    <mergeCell ref="E35:G35"/>
+    <mergeCell ref="H35:I35"/>
+    <mergeCell ref="A32:B32"/>
+    <mergeCell ref="C32:D32"/>
+    <mergeCell ref="E32:G32"/>
+    <mergeCell ref="H32:I32"/>
+    <mergeCell ref="A33:B33"/>
+    <mergeCell ref="C33:D33"/>
+    <mergeCell ref="E33:G33"/>
+    <mergeCell ref="H33:I33"/>
+    <mergeCell ref="A30:B30"/>
+    <mergeCell ref="C30:D30"/>
+    <mergeCell ref="E30:G30"/>
+    <mergeCell ref="H30:I30"/>
+    <mergeCell ref="A31:B31"/>
+    <mergeCell ref="C31:D31"/>
+    <mergeCell ref="E31:G31"/>
+    <mergeCell ref="H31:I31"/>
+    <mergeCell ref="A28:B28"/>
+    <mergeCell ref="C28:D28"/>
+    <mergeCell ref="E28:G28"/>
+    <mergeCell ref="H28:I28"/>
+    <mergeCell ref="A29:B29"/>
+    <mergeCell ref="C29:D29"/>
+    <mergeCell ref="E29:G29"/>
+    <mergeCell ref="H29:I29"/>
+    <mergeCell ref="A26:B26"/>
+    <mergeCell ref="C26:D26"/>
+    <mergeCell ref="E26:G26"/>
+    <mergeCell ref="H26:I26"/>
+    <mergeCell ref="A27:B27"/>
+    <mergeCell ref="C27:D27"/>
+    <mergeCell ref="E27:G27"/>
+    <mergeCell ref="H27:I27"/>
+    <mergeCell ref="A24:B24"/>
+    <mergeCell ref="C24:D24"/>
+    <mergeCell ref="E24:G24"/>
+    <mergeCell ref="H24:I24"/>
+    <mergeCell ref="A25:B25"/>
+    <mergeCell ref="C25:D25"/>
+    <mergeCell ref="E25:G25"/>
+    <mergeCell ref="H25:I25"/>
+    <mergeCell ref="A22:B22"/>
+    <mergeCell ref="C22:D22"/>
+    <mergeCell ref="E22:G22"/>
+    <mergeCell ref="H22:I22"/>
+    <mergeCell ref="A23:B23"/>
+    <mergeCell ref="C23:D23"/>
+    <mergeCell ref="E23:G23"/>
+    <mergeCell ref="H23:I23"/>
+    <mergeCell ref="A20:B20"/>
+    <mergeCell ref="C20:D20"/>
+    <mergeCell ref="E20:G20"/>
+    <mergeCell ref="H20:I20"/>
+    <mergeCell ref="A21:B21"/>
+    <mergeCell ref="C21:D21"/>
+    <mergeCell ref="E21:G21"/>
+    <mergeCell ref="H21:I21"/>
+    <mergeCell ref="A18:B18"/>
+    <mergeCell ref="C18:D18"/>
+    <mergeCell ref="E18:G18"/>
+    <mergeCell ref="H18:I18"/>
+    <mergeCell ref="A19:B19"/>
+    <mergeCell ref="C19:D19"/>
+    <mergeCell ref="E19:G19"/>
+    <mergeCell ref="H19:I19"/>
+    <mergeCell ref="A16:B16"/>
+    <mergeCell ref="C16:D16"/>
+    <mergeCell ref="E16:G16"/>
+    <mergeCell ref="H16:I16"/>
+    <mergeCell ref="A17:B17"/>
+    <mergeCell ref="C17:D17"/>
+    <mergeCell ref="E17:G17"/>
+    <mergeCell ref="H17:I17"/>
+    <mergeCell ref="A14:B14"/>
+    <mergeCell ref="C14:D14"/>
+    <mergeCell ref="E14:G14"/>
+    <mergeCell ref="H14:I14"/>
+    <mergeCell ref="A15:B15"/>
+    <mergeCell ref="C15:D15"/>
+    <mergeCell ref="E15:G15"/>
+    <mergeCell ref="H15:I15"/>
+    <mergeCell ref="A12:B12"/>
+    <mergeCell ref="C12:D12"/>
+    <mergeCell ref="E12:G12"/>
+    <mergeCell ref="H12:I12"/>
+    <mergeCell ref="A13:B13"/>
+    <mergeCell ref="C13:D13"/>
+    <mergeCell ref="E13:G13"/>
+    <mergeCell ref="H13:I13"/>
+    <mergeCell ref="A10:B10"/>
+    <mergeCell ref="C10:D10"/>
+    <mergeCell ref="E10:G10"/>
+    <mergeCell ref="H10:I10"/>
+    <mergeCell ref="A11:B11"/>
+    <mergeCell ref="C11:D11"/>
+    <mergeCell ref="E11:G11"/>
+    <mergeCell ref="H11:I11"/>
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="C4:E4"/>
+    <mergeCell ref="F4:I4"/>
+    <mergeCell ref="A9:B9"/>
+    <mergeCell ref="C9:D9"/>
+    <mergeCell ref="E9:G9"/>
+    <mergeCell ref="H9:I9"/>
+    <mergeCell ref="A8:B8"/>
+    <mergeCell ref="C8:D8"/>
+    <mergeCell ref="D2:E2"/>
+    <mergeCell ref="E8:G8"/>
+    <mergeCell ref="H8:I8"/>
+    <mergeCell ref="F5:I5"/>
+    <mergeCell ref="A5:B5"/>
+    <mergeCell ref="C5:E5"/>
+    <mergeCell ref="B3:D3"/>
+  </mergeCells>
+  <printOptions gridLines="false" gridLinesSet="true"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="1" orientation="default" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Skladová karta Excel: druhý list pro duplex (šablona + export).
Strana 1/2 ve šabloně (clone layoutu), export zapisuje jen hodnoty — bez kopírování stylů v PHP. Deník až 80 řádků.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/deploy/excel/skladova-karta.template.xlsx
+++ b/deploy/excel/skladova-karta.template.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xml:space="preserve">
   <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
-  <workbookPr defaultThemeVersion="124226"/>
+  <workbookPr codeName="ThisWorkbook"/>
   <bookViews>
-    <workbookView xWindow="120" yWindow="90" windowWidth="25815" windowHeight="11010"/>
+    <workbookView activeTab="0" autoFilterDateGrouping="true" firstSheet="0" minimized="false" showHorizontalScroll="true" showSheetTabs="true" showVerticalScroll="true" tabRatio="600" visibility="visible"/>
   </bookViews>
   <sheets>
-    <sheet name="Лист1" sheetId="1" r:id="rId1"/>
-    <sheet name="Лист2" sheetId="2" r:id="rId2"/>
-    <sheet name="Лист3" sheetId="3" r:id="rId3"/>
+    <sheet name="Strana 1" sheetId="1" r:id="rId4"/>
+    <sheet name="Strana 2" sheetId="2" r:id="rId5"/>
   </sheets>
-  <calcPr calcId="124519"/>
+  <definedNames/>
+  <calcPr calcId="999999" calcMode="auto" calcCompleted="1" fullCalcOnLoad="0" forceFullCalc="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="15">
   <si>
     <t>SKLADOVÁ KARTA - OPTIKA</t>
   </si>
@@ -24,19 +24,10 @@
     <t>DATUM NASKLADNĚNÍ :</t>
   </si>
   <si>
-    <t>CELKOVÁ METRÁŽ</t>
-  </si>
-  <si>
     <t>POČET VLÁKEN:</t>
   </si>
   <si>
-    <t>POČÁTEČNÍ STAV</t>
-  </si>
-  <si>
-    <t>TYP OK:</t>
-  </si>
-  <si>
-    <t>POZNÁMKA:</t>
+    <t>4 vl</t>
   </si>
   <si>
     <t>ŠARŽE:</t>
@@ -45,35 +36,45 @@
     <t>450-020858</t>
   </si>
   <si>
+    <t>TYP OK:</t>
+  </si>
+  <si>
     <r>
       <t xml:space="preserve">MLT  DROP  </t>
     </r>
     <r>
       <rPr>
-        <u/>
+        <rFont val="Calibri"/>
+        <b val="false"/>
+        <i val="false"/>
+        <strike val="false"/>
+        <color rgb="FF000000"/>
         <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="minor"/>
+        <u val="single"/>
       </rPr>
-      <t>BLOWN</t>
+      <t xml:space="preserve">BLOWN</t>
     </r>
     <r>
       <rPr>
+        <rFont val="Calibri"/>
+        <b val="false"/>
+        <i val="false"/>
+        <strike val="false"/>
+        <color rgb="FF000000"/>
         <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="minor"/>
+        <u val="none"/>
       </rPr>
       <t xml:space="preserve">  FLAT</t>
     </r>
   </si>
   <si>
-    <t>4 vl</t>
+    <t>CELKOVÁ METRÁŽ</t>
+  </si>
+  <si>
+    <t>POČÁTEČNÍ STAV</t>
+  </si>
+  <si>
+    <t>POZNÁMKA:</t>
   </si>
   <si>
     <t>DATUM</t>
@@ -91,103 +92,80 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xml:space="preserve">
   <numFmts count="2">
-    <numFmt numFmtId="44" formatCode="_-* #,##0.00\ &quot;₴&quot;_-;\-* #,##0.00\ &quot;₴&quot;_-;_-* &quot;-&quot;??\ &quot;₴&quot;_-;_-@_-"/>
-    <numFmt numFmtId="164" formatCode="#,##0.0\ _₴"/>
+    <numFmt numFmtId="164" formatCode="_-* #,##0.00\ &quot;₴&quot;_-;\-* #,##0.00\ &quot;₴&quot;_-;_-* &quot;-&quot;??\ &quot;₴&quot;_-;_-@_-"/>
+    <numFmt numFmtId="165" formatCode="#,##0.0\ _₴"/>
   </numFmts>
-  <fonts count="11">
+  <fonts count="7">
     <font>
+      <b val="0"/>
+      <i val="0"/>
+      <strike val="0"/>
+      <u val="none"/>
       <sz val="11"/>
-      <color theme="1"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
-      <family val="2"/>
-      <charset val="1"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
+      <b val="1"/>
+      <i val="0"/>
+      <strike val="0"/>
+      <u val="none"/>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
-      <family val="2"/>
-      <charset val="1"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="18"/>
-      <color theme="1"/>
+      <b val="1"/>
+      <i val="0"/>
+      <strike val="0"/>
+      <u val="none"/>
+      <sz val="20"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
-      <family val="2"/>
-      <charset val="204"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="20"/>
-      <color theme="1"/>
+      <b val="1"/>
+      <i val="0"/>
+      <strike val="0"/>
+      <u val="none"/>
+      <sz val="18"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
-      <family val="2"/>
-      <charset val="204"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
+      <b val="1"/>
+      <i val="0"/>
+      <strike val="0"/>
+      <u val="none"/>
       <sz val="22"/>
-      <color theme="1"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
-      <family val="2"/>
-      <charset val="204"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="12"/>
-      <color theme="1"/>
+      <b val="0"/>
+      <i val="0"/>
+      <strike val="0"/>
+      <u val="none"/>
+      <sz val="13"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
-      <family val="2"/>
-      <charset val="204"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
+      <b val="0"/>
+      <i val="0"/>
+      <strike val="0"/>
+      <u val="none"/>
+      <sz val="14"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
-      <family val="2"/>
-      <charset val="204"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <charset val="204"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="13"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <charset val="204"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="14"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <charset val="204"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="14"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <charset val="1"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -200,8 +178,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="0" tint="-0.249977111117893"/>
-        <bgColor indexed="64"/>
+        <fgColor rgb="FFBFBFBF"/>
+        <bgColor rgb="FFFFFFFF"/>
       </patternFill>
     </fill>
   </fills>
@@ -214,12 +192,87 @@
       <diagonal/>
     </border>
     <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
       <left style="thin">
-        <color indexed="64"/>
+        <color rgb="FF000000"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
       </left>
       <right/>
       <top style="thin">
-        <color indexed="64"/>
+        <color rgb="FF000000"/>
       </top>
       <bottom/>
       <diagonal/>
@@ -228,7 +281,7 @@
       <left/>
       <right/>
       <top style="thin">
-        <color indexed="64"/>
+        <color rgb="FF000000"/>
       </top>
       <bottom/>
       <diagonal/>
@@ -236,229 +289,152 @@
     <border>
       <left/>
       <right style="thin">
-        <color indexed="64"/>
+        <color rgb="FF000000"/>
       </right>
       <top style="thin">
-        <color indexed="64"/>
+        <color rgb="FF000000"/>
       </top>
       <bottom/>
       <diagonal/>
     </border>
     <border>
       <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
+        <color rgb="FF000000"/>
       </left>
       <right/>
       <top style="thin">
-        <color indexed="64"/>
+        <color rgb="FF000000"/>
       </top>
       <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
+        <color rgb="FF000000"/>
       </bottom>
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="41">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
-    <xf numFmtId="14" fontId="2" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="2" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="0" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
+    <xf xfId="0" fontId="0" numFmtId="164" fillId="0" borderId="0" applyFont="0" applyNumberFormat="1" applyFill="0" applyBorder="0" applyAlignment="0"/>
+    <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="0" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
+    <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="1" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="0"/>
+    <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="2" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="0"/>
+    <xf xfId="0" fontId="1" numFmtId="0" fillId="0" borderId="1" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="1" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="2" numFmtId="0" fillId="0" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="2" numFmtId="0" fillId="0" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="1">
+      <alignment vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="2" numFmtId="0" fillId="0" borderId="2" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="3" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="0"/>
+    <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="4" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="0"/>
+    <xf xfId="0" fontId="3" numFmtId="14" fillId="0" borderId="1" applyFont="1" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="3" numFmtId="14" fillId="0" borderId="2" applyFont="1" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="2" numFmtId="165" fillId="0" borderId="5" applyFont="1" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="2" numFmtId="165" fillId="0" borderId="6" applyFont="1" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="2" numFmtId="165" fillId="0" borderId="7" applyFont="1" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="3" numFmtId="0" fillId="0" borderId="5" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="3" numFmtId="0" fillId="0" borderId="7" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="2" numFmtId="0" fillId="0" borderId="5" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="2" numFmtId="0" fillId="0" borderId="6" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="2" numFmtId="0" fillId="0" borderId="7" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="2" numFmtId="0" fillId="0" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="4" numFmtId="164" fillId="0" borderId="0" applyFont="1" applyNumberFormat="1" applyFill="0" applyBorder="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="8" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="9" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="10" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="4" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="0" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="0" numFmtId="0" fillId="2" borderId="4" applyFont="0" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="0" numFmtId="0" fillId="2" borderId="0" applyFont="0" applyNumberFormat="0" applyFill="1" applyBorder="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="5" numFmtId="0" fillId="0" borderId="11" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="5" numFmtId="0" fillId="0" borderId="5" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="5" numFmtId="0" fillId="0" borderId="8" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="5" numFmtId="0" fillId="0" borderId="10" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="5" numFmtId="0" fillId="0" borderId="11" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="5" numFmtId="0" fillId="0" borderId="9" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="6" numFmtId="0" fillId="2" borderId="4" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="6" numFmtId="0" fillId="2" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="6" numFmtId="0" fillId="2" borderId="4" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="6" numFmtId="0" fillId="2" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
     </xf>
   </cellXfs>
-  <cellStyles count="2">
-    <cellStyle name="Денежный" xfId="1" builtinId="4"/>
-    <cellStyle name="Обычный" xfId="0" builtinId="0"/>
+  <cellStyles count="1">
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <tableStyles defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotTableStyle1"/>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Тема Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Стандартная">
       <a:dk1>
@@ -568,7 +544,7 @@
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Стандартная">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -741,22 +717,25 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xml:space="preserve" mc:Ignorable="x14ac">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+  </sheetPr>
   <dimension ref="A1:L48"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col min="1" max="1" width="9.28515625" customWidth="1"/>
-    <col min="2" max="2" width="10.28515625" customWidth="1"/>
-    <col min="4" max="4" width="13" customWidth="1"/>
-    <col min="5" max="5" width="7.28515625" customWidth="1"/>
-    <col min="6" max="6" width="9.28515625" customWidth="1"/>
-    <col min="7" max="7" width="6.7109375" customWidth="1"/>
-    <col min="8" max="8" width="6.85546875" customWidth="1"/>
-    <col min="9" max="9" width="16.42578125" customWidth="1"/>
-    <col min="10" max="10" width="1" customWidth="1"/>
+    <col min="1" max="1" width="9.28515625" customWidth="true" style="0"/>
+    <col min="2" max="2" width="10.28515625" customWidth="true" style="0"/>
+    <col min="4" max="4" width="13" customWidth="true" style="0"/>
+    <col min="5" max="5" width="7.28515625" customWidth="true" style="0"/>
+    <col min="6" max="6" width="9.28515625" customWidth="true" style="0"/>
+    <col min="7" max="7" width="6.7109375" customWidth="true" style="0"/>
+    <col min="8" max="8" width="6.85546875" customWidth="true" style="0"/>
+    <col min="9" max="9" width="16.42578125" customWidth="true" style="0"/>
+    <col min="10" max="10" width="1" customWidth="true" style="0"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="28.5">
+    <row r="1" spans="1:12" customHeight="1" ht="28.5">
       <c r="A1" s="23" t="s">
         <v>0</v>
       </c>
@@ -772,7 +751,7 @@
       <c r="K1" s="1"/>
       <c r="L1" s="1"/>
     </row>
-    <row r="2" spans="1:12" ht="33" customHeight="1">
+    <row r="2" spans="1:12" customHeight="1" ht="33">
       <c r="A2" s="31" t="s">
         <v>1</v>
       </c>
@@ -783,54 +762,54 @@
       </c>
       <c r="E2" s="13"/>
       <c r="F2" s="31" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G2" s="5"/>
       <c r="H2" s="3"/>
       <c r="I2" s="9" t="s">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="J2" s="8"/>
       <c r="K2" s="8"/>
     </row>
-    <row r="3" spans="1:12" ht="33.75" customHeight="1">
+    <row r="3" spans="1:12" customHeight="1" ht="33.75">
       <c r="A3" s="32" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="B3" s="22" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="C3" s="22"/>
       <c r="D3" s="22"/>
       <c r="E3" s="7"/>
       <c r="F3" s="35" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G3" s="5"/>
       <c r="H3" s="6" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="I3" s="4"/>
       <c r="J3" s="11"/>
     </row>
-    <row r="4" spans="1:12" ht="26.25" customHeight="1">
+    <row r="4" spans="1:12" customHeight="1" ht="26.25">
       <c r="A4" s="33" t="s">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="B4" s="34"/>
       <c r="C4" s="33" t="s">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D4" s="36"/>
       <c r="E4" s="34"/>
       <c r="F4" s="24" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="G4" s="25"/>
       <c r="H4" s="25"/>
       <c r="I4" s="26"/>
     </row>
-    <row r="5" spans="1:12" ht="35.25" customHeight="1">
+    <row r="5" spans="1:12" customHeight="1" ht="35.25">
       <c r="A5" s="17">
         <v>2100</v>
       </c>
@@ -847,7 +826,7 @@
       <c r="H5" s="15"/>
       <c r="I5" s="16"/>
     </row>
-    <row r="6" spans="1:12" ht="9" customHeight="1" thickBot="1">
+    <row r="6" spans="1:12" customHeight="1" ht="9">
       <c r="A6" s="10"/>
       <c r="B6" s="10"/>
       <c r="C6" s="10"/>
@@ -858,10 +837,10 @@
       <c r="H6" s="10"/>
       <c r="I6" s="10"/>
     </row>
-    <row r="7" spans="1:12" ht="12" customHeight="1">
+    <row r="7" spans="1:12" customHeight="1" ht="12">
       <c r="I7" s="2"/>
     </row>
-    <row r="8" spans="1:12" ht="32.1" customHeight="1">
+    <row r="8" spans="1:12" customHeight="1" ht="32.1">
       <c r="A8" s="39" t="s">
         <v>11</v>
       </c>
@@ -881,7 +860,7 @@
       <c r="I8" s="38"/>
       <c r="J8" s="11"/>
     </row>
-    <row r="9" spans="1:12" ht="32.1" customHeight="1">
+    <row r="9" spans="1:12" customHeight="1" ht="32.1">
       <c r="A9" s="27"/>
       <c r="B9" s="28"/>
       <c r="C9" s="27"/>
@@ -893,7 +872,7 @@
       <c r="I9" s="28"/>
       <c r="J9" s="11"/>
     </row>
-    <row r="10" spans="1:12" ht="32.1" customHeight="1">
+    <row r="10" spans="1:12" customHeight="1" ht="32.1">
       <c r="A10" s="29"/>
       <c r="B10" s="30"/>
       <c r="C10" s="29"/>
@@ -905,7 +884,7 @@
       <c r="I10" s="30"/>
       <c r="J10" s="11"/>
     </row>
-    <row r="11" spans="1:12" ht="32.1" customHeight="1">
+    <row r="11" spans="1:12" customHeight="1" ht="32.1">
       <c r="A11" s="27"/>
       <c r="B11" s="28"/>
       <c r="C11" s="27"/>
@@ -917,7 +896,7 @@
       <c r="I11" s="28"/>
       <c r="J11" s="11"/>
     </row>
-    <row r="12" spans="1:12" ht="32.1" customHeight="1">
+    <row r="12" spans="1:12" customHeight="1" ht="32.1">
       <c r="A12" s="29"/>
       <c r="B12" s="30"/>
       <c r="C12" s="29"/>
@@ -929,7 +908,7 @@
       <c r="I12" s="30"/>
       <c r="J12" s="11"/>
     </row>
-    <row r="13" spans="1:12" ht="32.1" customHeight="1">
+    <row r="13" spans="1:12" customHeight="1" ht="32.1">
       <c r="A13" s="27"/>
       <c r="B13" s="28"/>
       <c r="C13" s="27"/>
@@ -941,7 +920,7 @@
       <c r="I13" s="28"/>
       <c r="J13" s="11"/>
     </row>
-    <row r="14" spans="1:12" ht="32.1" customHeight="1">
+    <row r="14" spans="1:12" customHeight="1" ht="32.1">
       <c r="A14" s="29"/>
       <c r="B14" s="30"/>
       <c r="C14" s="29"/>
@@ -953,7 +932,7 @@
       <c r="I14" s="30"/>
       <c r="J14" s="11"/>
     </row>
-    <row r="15" spans="1:12" ht="32.1" customHeight="1">
+    <row r="15" spans="1:12" customHeight="1" ht="32.1">
       <c r="A15" s="27"/>
       <c r="B15" s="28"/>
       <c r="C15" s="27"/>
@@ -965,7 +944,7 @@
       <c r="I15" s="28"/>
       <c r="J15" s="11"/>
     </row>
-    <row r="16" spans="1:12" ht="32.1" customHeight="1">
+    <row r="16" spans="1:12" customHeight="1" ht="32.1">
       <c r="A16" s="29"/>
       <c r="B16" s="30"/>
       <c r="C16" s="29"/>
@@ -977,7 +956,7 @@
       <c r="I16" s="30"/>
       <c r="J16" s="11"/>
     </row>
-    <row r="17" spans="1:10" ht="32.1" customHeight="1">
+    <row r="17" spans="1:12" customHeight="1" ht="32.1">
       <c r="A17" s="27"/>
       <c r="B17" s="28"/>
       <c r="C17" s="27"/>
@@ -989,7 +968,7 @@
       <c r="I17" s="28"/>
       <c r="J17" s="11"/>
     </row>
-    <row r="18" spans="1:10" ht="32.1" customHeight="1">
+    <row r="18" spans="1:12" customHeight="1" ht="32.1">
       <c r="A18" s="29"/>
       <c r="B18" s="30"/>
       <c r="C18" s="29"/>
@@ -1001,7 +980,7 @@
       <c r="I18" s="30"/>
       <c r="J18" s="11"/>
     </row>
-    <row r="19" spans="1:10" ht="32.1" customHeight="1">
+    <row r="19" spans="1:12" customHeight="1" ht="32.1">
       <c r="A19" s="27"/>
       <c r="B19" s="28"/>
       <c r="C19" s="27"/>
@@ -1013,7 +992,7 @@
       <c r="I19" s="28"/>
       <c r="J19" s="11"/>
     </row>
-    <row r="20" spans="1:10" ht="32.1" customHeight="1">
+    <row r="20" spans="1:12" customHeight="1" ht="32.1">
       <c r="A20" s="29"/>
       <c r="B20" s="30"/>
       <c r="C20" s="29"/>
@@ -1025,7 +1004,7 @@
       <c r="I20" s="30"/>
       <c r="J20" s="11"/>
     </row>
-    <row r="21" spans="1:10" ht="32.1" customHeight="1">
+    <row r="21" spans="1:12" customHeight="1" ht="32.1">
       <c r="A21" s="27"/>
       <c r="B21" s="28"/>
       <c r="C21" s="27"/>
@@ -1037,7 +1016,7 @@
       <c r="I21" s="28"/>
       <c r="J21" s="11"/>
     </row>
-    <row r="22" spans="1:10" ht="32.1" customHeight="1">
+    <row r="22" spans="1:12" customHeight="1" ht="32.1">
       <c r="A22" s="29"/>
       <c r="B22" s="30"/>
       <c r="C22" s="29"/>
@@ -1049,7 +1028,7 @@
       <c r="I22" s="30"/>
       <c r="J22" s="11"/>
     </row>
-    <row r="23" spans="1:10" ht="32.1" customHeight="1">
+    <row r="23" spans="1:12" customHeight="1" ht="32.1">
       <c r="A23" s="27"/>
       <c r="B23" s="28"/>
       <c r="C23" s="27"/>
@@ -1061,7 +1040,7 @@
       <c r="I23" s="28"/>
       <c r="J23" s="11"/>
     </row>
-    <row r="24" spans="1:10" ht="32.1" customHeight="1">
+    <row r="24" spans="1:12" customHeight="1" ht="32.1">
       <c r="A24" s="29"/>
       <c r="B24" s="30"/>
       <c r="C24" s="29"/>
@@ -1073,7 +1052,7 @@
       <c r="I24" s="30"/>
       <c r="J24" s="11"/>
     </row>
-    <row r="25" spans="1:10" ht="32.1" customHeight="1">
+    <row r="25" spans="1:12" customHeight="1" ht="32.1">
       <c r="A25" s="27"/>
       <c r="B25" s="28"/>
       <c r="C25" s="27"/>
@@ -1085,27 +1064,19 @@
       <c r="I25" s="28"/>
       <c r="J25" s="11"/>
     </row>
-    <row r="26" spans="1:10" ht="32.1" customHeight="1">
-      <c r="A26" s="37" t="s">
-        <v>11</v>
-      </c>
+    <row r="26" spans="1:12" customHeight="1" ht="32.1">
+      <c r="A26" s="37"/>
       <c r="B26" s="38"/>
-      <c r="C26" s="37" t="s">
-        <v>12</v>
-      </c>
+      <c r="C26" s="37"/>
       <c r="D26" s="38"/>
-      <c r="E26" s="37" t="s">
-        <v>13</v>
-      </c>
+      <c r="E26" s="37"/>
       <c r="F26" s="38"/>
       <c r="G26" s="38"/>
-      <c r="H26" s="37" t="s">
-        <v>14</v>
-      </c>
+      <c r="H26" s="37"/>
       <c r="I26" s="38"/>
       <c r="J26" s="11"/>
     </row>
-    <row r="27" spans="1:10" ht="32.1" customHeight="1">
+    <row r="27" spans="1:12" customHeight="1" ht="32.1">
       <c r="A27" s="27"/>
       <c r="B27" s="28"/>
       <c r="C27" s="27"/>
@@ -1117,7 +1088,7 @@
       <c r="I27" s="28"/>
       <c r="J27" s="11"/>
     </row>
-    <row r="28" spans="1:10" ht="32.1" customHeight="1">
+    <row r="28" spans="1:12" customHeight="1" ht="32.1">
       <c r="A28" s="29"/>
       <c r="B28" s="30"/>
       <c r="C28" s="29"/>
@@ -1129,7 +1100,7 @@
       <c r="I28" s="30"/>
       <c r="J28" s="11"/>
     </row>
-    <row r="29" spans="1:10" ht="32.1" customHeight="1">
+    <row r="29" spans="1:12" customHeight="1" ht="32.1">
       <c r="A29" s="27"/>
       <c r="B29" s="28"/>
       <c r="C29" s="27"/>
@@ -1141,7 +1112,7 @@
       <c r="I29" s="28"/>
       <c r="J29" s="11"/>
     </row>
-    <row r="30" spans="1:10" ht="32.1" customHeight="1">
+    <row r="30" spans="1:12" customHeight="1" ht="32.1">
       <c r="A30" s="29"/>
       <c r="B30" s="30"/>
       <c r="C30" s="29"/>
@@ -1153,7 +1124,7 @@
       <c r="I30" s="30"/>
       <c r="J30" s="11"/>
     </row>
-    <row r="31" spans="1:10" ht="32.1" customHeight="1">
+    <row r="31" spans="1:12" customHeight="1" ht="32.1">
       <c r="A31" s="27"/>
       <c r="B31" s="28"/>
       <c r="C31" s="27"/>
@@ -1165,7 +1136,7 @@
       <c r="I31" s="28"/>
       <c r="J31" s="11"/>
     </row>
-    <row r="32" spans="1:10" ht="32.1" customHeight="1">
+    <row r="32" spans="1:12" customHeight="1" ht="32.1">
       <c r="A32" s="29"/>
       <c r="B32" s="30"/>
       <c r="C32" s="29"/>
@@ -1177,7 +1148,7 @@
       <c r="I32" s="30"/>
       <c r="J32" s="11"/>
     </row>
-    <row r="33" spans="1:10" ht="32.1" customHeight="1">
+    <row r="33" spans="1:12" customHeight="1" ht="32.1">
       <c r="A33" s="27"/>
       <c r="B33" s="28"/>
       <c r="C33" s="27"/>
@@ -1189,7 +1160,7 @@
       <c r="I33" s="28"/>
       <c r="J33" s="11"/>
     </row>
-    <row r="34" spans="1:10" ht="32.1" customHeight="1">
+    <row r="34" spans="1:12" customHeight="1" ht="32.1">
       <c r="A34" s="29"/>
       <c r="B34" s="30"/>
       <c r="C34" s="29"/>
@@ -1201,7 +1172,7 @@
       <c r="I34" s="30"/>
       <c r="J34" s="11"/>
     </row>
-    <row r="35" spans="1:10" ht="32.1" customHeight="1">
+    <row r="35" spans="1:12" customHeight="1" ht="32.1">
       <c r="A35" s="27"/>
       <c r="B35" s="28"/>
       <c r="C35" s="27"/>
@@ -1213,7 +1184,7 @@
       <c r="I35" s="28"/>
       <c r="J35" s="11"/>
     </row>
-    <row r="36" spans="1:10" ht="32.1" customHeight="1">
+    <row r="36" spans="1:12" customHeight="1" ht="32.1">
       <c r="A36" s="29"/>
       <c r="B36" s="30"/>
       <c r="C36" s="29"/>
@@ -1225,7 +1196,7 @@
       <c r="I36" s="30"/>
       <c r="J36" s="11"/>
     </row>
-    <row r="37" spans="1:10" ht="32.1" customHeight="1">
+    <row r="37" spans="1:12" customHeight="1" ht="32.1">
       <c r="A37" s="27"/>
       <c r="B37" s="28"/>
       <c r="C37" s="27"/>
@@ -1237,7 +1208,7 @@
       <c r="I37" s="28"/>
       <c r="J37" s="11"/>
     </row>
-    <row r="38" spans="1:10" ht="32.1" customHeight="1">
+    <row r="38" spans="1:12" customHeight="1" ht="32.1">
       <c r="A38" s="29"/>
       <c r="B38" s="30"/>
       <c r="C38" s="29"/>
@@ -1249,7 +1220,7 @@
       <c r="I38" s="30"/>
       <c r="J38" s="11"/>
     </row>
-    <row r="39" spans="1:10" ht="32.1" customHeight="1">
+    <row r="39" spans="1:12" customHeight="1" ht="32.1">
       <c r="A39" s="27"/>
       <c r="B39" s="28"/>
       <c r="C39" s="27"/>
@@ -1261,7 +1232,7 @@
       <c r="I39" s="28"/>
       <c r="J39" s="11"/>
     </row>
-    <row r="40" spans="1:10" ht="32.1" customHeight="1">
+    <row r="40" spans="1:12" customHeight="1" ht="32.1">
       <c r="A40" s="29"/>
       <c r="B40" s="30"/>
       <c r="C40" s="29"/>
@@ -1273,7 +1244,7 @@
       <c r="I40" s="30"/>
       <c r="J40" s="11"/>
     </row>
-    <row r="41" spans="1:10" ht="32.1" customHeight="1">
+    <row r="41" spans="1:12" customHeight="1" ht="32.1">
       <c r="A41" s="27"/>
       <c r="B41" s="28"/>
       <c r="C41" s="27"/>
@@ -1285,7 +1256,7 @@
       <c r="I41" s="28"/>
       <c r="J41" s="11"/>
     </row>
-    <row r="42" spans="1:10" ht="32.1" customHeight="1">
+    <row r="42" spans="1:12" customHeight="1" ht="32.1">
       <c r="A42" s="29"/>
       <c r="B42" s="30"/>
       <c r="C42" s="29"/>
@@ -1297,7 +1268,7 @@
       <c r="I42" s="30"/>
       <c r="J42" s="11"/>
     </row>
-    <row r="43" spans="1:10" ht="32.1" customHeight="1">
+    <row r="43" spans="1:12" customHeight="1" ht="32.1">
       <c r="A43" s="27"/>
       <c r="B43" s="28"/>
       <c r="C43" s="27"/>
@@ -1309,7 +1280,7 @@
       <c r="I43" s="28"/>
       <c r="J43" s="11"/>
     </row>
-    <row r="44" spans="1:10" ht="32.1" customHeight="1">
+    <row r="44" spans="1:12" customHeight="1" ht="32.1">
       <c r="A44" s="29"/>
       <c r="B44" s="30"/>
       <c r="C44" s="29"/>
@@ -1321,7 +1292,7 @@
       <c r="I44" s="30"/>
       <c r="J44" s="11"/>
     </row>
-    <row r="45" spans="1:10" ht="32.1" customHeight="1">
+    <row r="45" spans="1:12" customHeight="1" ht="32.1">
       <c r="A45" s="27"/>
       <c r="B45" s="28"/>
       <c r="C45" s="27"/>
@@ -1333,7 +1304,7 @@
       <c r="I45" s="28"/>
       <c r="J45" s="11"/>
     </row>
-    <row r="46" spans="1:10" ht="32.1" customHeight="1">
+    <row r="46" spans="1:12" customHeight="1" ht="32.1">
       <c r="A46" s="29"/>
       <c r="B46" s="30"/>
       <c r="C46" s="29"/>
@@ -1345,7 +1316,7 @@
       <c r="I46" s="30"/>
       <c r="J46" s="11"/>
     </row>
-    <row r="47" spans="1:10" ht="32.1" customHeight="1">
+    <row r="47" spans="1:12" customHeight="1" ht="32.1">
       <c r="A47" s="27"/>
       <c r="B47" s="28"/>
       <c r="C47" s="27"/>
@@ -1357,7 +1328,7 @@
       <c r="I47" s="28"/>
       <c r="J47" s="11"/>
     </row>
-    <row r="48" spans="1:10" ht="32.1" customHeight="1">
+    <row r="48" spans="1:12" customHeight="1" ht="32.1">
       <c r="A48" s="29"/>
       <c r="B48" s="30"/>
       <c r="C48" s="29"/>
@@ -1370,7 +1341,7 @@
       <c r="J48" s="11"/>
     </row>
   </sheetData>
-  <mergeCells count="173">
+  <mergeCells>
     <mergeCell ref="A48:B48"/>
     <mergeCell ref="C48:D48"/>
     <mergeCell ref="E48:G48"/>
@@ -1545,25 +1516,814 @@
     <mergeCell ref="C5:E5"/>
     <mergeCell ref="B3:D3"/>
   </mergeCells>
-  <pageMargins left="0.70866141732283472" right="0.51181102362204722" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <printOptions gridLines="false" gridLinesSet="true"/>
+  <pageMargins left="0.70866141732283" right="0.51181102362205" top="0.74803149606299" bottom="0.74803149606299" header="0.31496062992126" footer="0.31496062992126"/>
+  <pageSetup paperSize="9" orientation="portrait" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" r:id="rId1ps"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xml:space="preserve" mc:Ignorable="x14ac">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+  </sheetPr>
+  <dimension ref="A1:L48"/>
+  <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col min="1" max="1" width="9.28515625" customWidth="true" style="0"/>
+    <col min="2" max="2" width="10.28515625" customWidth="true" style="0"/>
+    <col min="4" max="4" width="13" customWidth="true" style="0"/>
+    <col min="5" max="5" width="7.28515625" customWidth="true" style="0"/>
+    <col min="6" max="6" width="9.28515625" customWidth="true" style="0"/>
+    <col min="7" max="7" width="6.7109375" customWidth="true" style="0"/>
+    <col min="8" max="8" width="6.85546875" customWidth="true" style="0"/>
+    <col min="9" max="9" width="16.42578125" customWidth="true" style="0"/>
+    <col min="10" max="10" width="1" customWidth="true" style="0"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:12" customHeight="1" ht="28.5">
+      <c r="A1" s="23" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="23"/>
+      <c r="C1" s="23"/>
+      <c r="D1" s="23"/>
+      <c r="E1" s="23"/>
+      <c r="F1" s="23"/>
+      <c r="G1" s="23"/>
+      <c r="H1" s="23"/>
+      <c r="I1" s="23"/>
+      <c r="J1" s="1"/>
+      <c r="K1" s="1"/>
+      <c r="L1" s="1"/>
+    </row>
+    <row r="2" spans="1:12" customHeight="1" ht="33">
+      <c r="A2" s="31" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="12">
+        <v>46167</v>
+      </c>
+      <c r="E2" s="13"/>
+      <c r="F2" s="31" t="s">
+        <v>2</v>
+      </c>
+      <c r="G2" s="5"/>
+      <c r="H2" s="3"/>
+      <c r="I2" s="9" t="s">
+        <v>3</v>
+      </c>
+      <c r="J2" s="8"/>
+      <c r="K2" s="8"/>
+    </row>
+    <row r="3" spans="1:12" customHeight="1" ht="33.75">
+      <c r="A3" s="32" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" s="22" t="s">
+        <v>5</v>
+      </c>
+      <c r="C3" s="22"/>
+      <c r="D3" s="22"/>
+      <c r="E3" s="7"/>
+      <c r="F3" s="35" t="s">
+        <v>6</v>
+      </c>
+      <c r="G3" s="5"/>
+      <c r="H3" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="I3" s="4"/>
+      <c r="J3" s="11"/>
+    </row>
+    <row r="4" spans="1:12" customHeight="1" ht="26.25">
+      <c r="A4" s="33" t="s">
+        <v>8</v>
+      </c>
+      <c r="B4" s="34"/>
+      <c r="C4" s="33" t="s">
+        <v>9</v>
+      </c>
+      <c r="D4" s="36"/>
+      <c r="E4" s="34"/>
+      <c r="F4" s="24" t="s">
+        <v>10</v>
+      </c>
+      <c r="G4" s="25"/>
+      <c r="H4" s="25"/>
+      <c r="I4" s="26"/>
+    </row>
+    <row r="5" spans="1:12" customHeight="1" ht="35.25">
+      <c r="A5" s="17">
+        <v>2100</v>
+      </c>
+      <c r="B5" s="18"/>
+      <c r="C5" s="19">
+        <v>4500</v>
+      </c>
+      <c r="D5" s="20"/>
+      <c r="E5" s="21"/>
+      <c r="F5" s="14">
+        <v>2</v>
+      </c>
+      <c r="G5" s="15"/>
+      <c r="H5" s="15"/>
+      <c r="I5" s="16"/>
+    </row>
+    <row r="6" spans="1:12" customHeight="1" ht="9">
+      <c r="A6" s="10"/>
+      <c r="B6" s="10"/>
+      <c r="C6" s="10"/>
+      <c r="D6" s="10"/>
+      <c r="E6" s="10"/>
+      <c r="F6" s="10"/>
+      <c r="G6" s="10"/>
+      <c r="H6" s="10"/>
+      <c r="I6" s="10"/>
+    </row>
+    <row r="7" spans="1:12" customHeight="1" ht="12">
+      <c r="I7" s="2"/>
+    </row>
+    <row r="8" spans="1:12" customHeight="1" ht="32.1">
+      <c r="A8" s="39" t="s">
+        <v>11</v>
+      </c>
+      <c r="B8" s="40"/>
+      <c r="C8" s="37" t="s">
+        <v>12</v>
+      </c>
+      <c r="D8" s="38"/>
+      <c r="E8" s="37" t="s">
+        <v>13</v>
+      </c>
+      <c r="F8" s="38"/>
+      <c r="G8" s="38"/>
+      <c r="H8" s="37" t="s">
+        <v>14</v>
+      </c>
+      <c r="I8" s="38"/>
+      <c r="J8" s="11"/>
+    </row>
+    <row r="9" spans="1:12" customHeight="1" ht="32.1">
+      <c r="A9" s="27"/>
+      <c r="B9" s="28"/>
+      <c r="C9" s="27"/>
+      <c r="D9" s="28"/>
+      <c r="E9" s="27"/>
+      <c r="F9" s="28"/>
+      <c r="G9" s="28"/>
+      <c r="H9" s="27"/>
+      <c r="I9" s="28"/>
+      <c r="J9" s="11"/>
+    </row>
+    <row r="10" spans="1:12" customHeight="1" ht="32.1">
+      <c r="A10" s="29"/>
+      <c r="B10" s="30"/>
+      <c r="C10" s="29"/>
+      <c r="D10" s="30"/>
+      <c r="E10" s="29"/>
+      <c r="F10" s="30"/>
+      <c r="G10" s="30"/>
+      <c r="H10" s="29"/>
+      <c r="I10" s="30"/>
+      <c r="J10" s="11"/>
+    </row>
+    <row r="11" spans="1:12" customHeight="1" ht="32.1">
+      <c r="A11" s="27"/>
+      <c r="B11" s="28"/>
+      <c r="C11" s="27"/>
+      <c r="D11" s="28"/>
+      <c r="E11" s="27"/>
+      <c r="F11" s="28"/>
+      <c r="G11" s="28"/>
+      <c r="H11" s="27"/>
+      <c r="I11" s="28"/>
+      <c r="J11" s="11"/>
+    </row>
+    <row r="12" spans="1:12" customHeight="1" ht="32.1">
+      <c r="A12" s="29"/>
+      <c r="B12" s="30"/>
+      <c r="C12" s="29"/>
+      <c r="D12" s="30"/>
+      <c r="E12" s="29"/>
+      <c r="F12" s="30"/>
+      <c r="G12" s="30"/>
+      <c r="H12" s="29"/>
+      <c r="I12" s="30"/>
+      <c r="J12" s="11"/>
+    </row>
+    <row r="13" spans="1:12" customHeight="1" ht="32.1">
+      <c r="A13" s="27"/>
+      <c r="B13" s="28"/>
+      <c r="C13" s="27"/>
+      <c r="D13" s="28"/>
+      <c r="E13" s="27"/>
+      <c r="F13" s="28"/>
+      <c r="G13" s="28"/>
+      <c r="H13" s="27"/>
+      <c r="I13" s="28"/>
+      <c r="J13" s="11"/>
+    </row>
+    <row r="14" spans="1:12" customHeight="1" ht="32.1">
+      <c r="A14" s="29"/>
+      <c r="B14" s="30"/>
+      <c r="C14" s="29"/>
+      <c r="D14" s="30"/>
+      <c r="E14" s="29"/>
+      <c r="F14" s="30"/>
+      <c r="G14" s="30"/>
+      <c r="H14" s="29"/>
+      <c r="I14" s="30"/>
+      <c r="J14" s="11"/>
+    </row>
+    <row r="15" spans="1:12" customHeight="1" ht="32.1">
+      <c r="A15" s="27"/>
+      <c r="B15" s="28"/>
+      <c r="C15" s="27"/>
+      <c r="D15" s="28"/>
+      <c r="E15" s="27"/>
+      <c r="F15" s="28"/>
+      <c r="G15" s="28"/>
+      <c r="H15" s="27"/>
+      <c r="I15" s="28"/>
+      <c r="J15" s="11"/>
+    </row>
+    <row r="16" spans="1:12" customHeight="1" ht="32.1">
+      <c r="A16" s="29"/>
+      <c r="B16" s="30"/>
+      <c r="C16" s="29"/>
+      <c r="D16" s="30"/>
+      <c r="E16" s="29"/>
+      <c r="F16" s="30"/>
+      <c r="G16" s="30"/>
+      <c r="H16" s="29"/>
+      <c r="I16" s="30"/>
+      <c r="J16" s="11"/>
+    </row>
+    <row r="17" spans="1:12" customHeight="1" ht="32.1">
+      <c r="A17" s="27"/>
+      <c r="B17" s="28"/>
+      <c r="C17" s="27"/>
+      <c r="D17" s="28"/>
+      <c r="E17" s="27"/>
+      <c r="F17" s="28"/>
+      <c r="G17" s="28"/>
+      <c r="H17" s="27"/>
+      <c r="I17" s="28"/>
+      <c r="J17" s="11"/>
+    </row>
+    <row r="18" spans="1:12" customHeight="1" ht="32.1">
+      <c r="A18" s="29"/>
+      <c r="B18" s="30"/>
+      <c r="C18" s="29"/>
+      <c r="D18" s="30"/>
+      <c r="E18" s="29"/>
+      <c r="F18" s="30"/>
+      <c r="G18" s="30"/>
+      <c r="H18" s="29"/>
+      <c r="I18" s="30"/>
+      <c r="J18" s="11"/>
+    </row>
+    <row r="19" spans="1:12" customHeight="1" ht="32.1">
+      <c r="A19" s="27"/>
+      <c r="B19" s="28"/>
+      <c r="C19" s="27"/>
+      <c r="D19" s="28"/>
+      <c r="E19" s="27"/>
+      <c r="F19" s="28"/>
+      <c r="G19" s="28"/>
+      <c r="H19" s="27"/>
+      <c r="I19" s="28"/>
+      <c r="J19" s="11"/>
+    </row>
+    <row r="20" spans="1:12" customHeight="1" ht="32.1">
+      <c r="A20" s="29"/>
+      <c r="B20" s="30"/>
+      <c r="C20" s="29"/>
+      <c r="D20" s="30"/>
+      <c r="E20" s="29"/>
+      <c r="F20" s="30"/>
+      <c r="G20" s="30"/>
+      <c r="H20" s="29"/>
+      <c r="I20" s="30"/>
+      <c r="J20" s="11"/>
+    </row>
+    <row r="21" spans="1:12" customHeight="1" ht="32.1">
+      <c r="A21" s="27"/>
+      <c r="B21" s="28"/>
+      <c r="C21" s="27"/>
+      <c r="D21" s="28"/>
+      <c r="E21" s="27"/>
+      <c r="F21" s="28"/>
+      <c r="G21" s="28"/>
+      <c r="H21" s="27"/>
+      <c r="I21" s="28"/>
+      <c r="J21" s="11"/>
+    </row>
+    <row r="22" spans="1:12" customHeight="1" ht="32.1">
+      <c r="A22" s="29"/>
+      <c r="B22" s="30"/>
+      <c r="C22" s="29"/>
+      <c r="D22" s="30"/>
+      <c r="E22" s="29"/>
+      <c r="F22" s="30"/>
+      <c r="G22" s="30"/>
+      <c r="H22" s="29"/>
+      <c r="I22" s="30"/>
+      <c r="J22" s="11"/>
+    </row>
+    <row r="23" spans="1:12" customHeight="1" ht="32.1">
+      <c r="A23" s="27"/>
+      <c r="B23" s="28"/>
+      <c r="C23" s="27"/>
+      <c r="D23" s="28"/>
+      <c r="E23" s="27"/>
+      <c r="F23" s="28"/>
+      <c r="G23" s="28"/>
+      <c r="H23" s="27"/>
+      <c r="I23" s="28"/>
+      <c r="J23" s="11"/>
+    </row>
+    <row r="24" spans="1:12" customHeight="1" ht="32.1">
+      <c r="A24" s="29"/>
+      <c r="B24" s="30"/>
+      <c r="C24" s="29"/>
+      <c r="D24" s="30"/>
+      <c r="E24" s="29"/>
+      <c r="F24" s="30"/>
+      <c r="G24" s="30"/>
+      <c r="H24" s="29"/>
+      <c r="I24" s="30"/>
+      <c r="J24" s="11"/>
+    </row>
+    <row r="25" spans="1:12" customHeight="1" ht="32.1">
+      <c r="A25" s="27"/>
+      <c r="B25" s="28"/>
+      <c r="C25" s="27"/>
+      <c r="D25" s="28"/>
+      <c r="E25" s="27"/>
+      <c r="F25" s="28"/>
+      <c r="G25" s="28"/>
+      <c r="H25" s="27"/>
+      <c r="I25" s="28"/>
+      <c r="J25" s="11"/>
+    </row>
+    <row r="26" spans="1:12" customHeight="1" ht="32.1">
+      <c r="A26" s="37"/>
+      <c r="B26" s="38"/>
+      <c r="C26" s="37"/>
+      <c r="D26" s="38"/>
+      <c r="E26" s="37"/>
+      <c r="F26" s="38"/>
+      <c r="G26" s="38"/>
+      <c r="H26" s="37"/>
+      <c r="I26" s="38"/>
+      <c r="J26" s="11"/>
+    </row>
+    <row r="27" spans="1:12" customHeight="1" ht="32.1">
+      <c r="A27" s="27"/>
+      <c r="B27" s="28"/>
+      <c r="C27" s="27"/>
+      <c r="D27" s="28"/>
+      <c r="E27" s="27"/>
+      <c r="F27" s="28"/>
+      <c r="G27" s="28"/>
+      <c r="H27" s="27"/>
+      <c r="I27" s="28"/>
+      <c r="J27" s="11"/>
+    </row>
+    <row r="28" spans="1:12" customHeight="1" ht="32.1">
+      <c r="A28" s="29"/>
+      <c r="B28" s="30"/>
+      <c r="C28" s="29"/>
+      <c r="D28" s="30"/>
+      <c r="E28" s="29"/>
+      <c r="F28" s="30"/>
+      <c r="G28" s="30"/>
+      <c r="H28" s="29"/>
+      <c r="I28" s="30"/>
+      <c r="J28" s="11"/>
+    </row>
+    <row r="29" spans="1:12" customHeight="1" ht="32.1">
+      <c r="A29" s="27"/>
+      <c r="B29" s="28"/>
+      <c r="C29" s="27"/>
+      <c r="D29" s="28"/>
+      <c r="E29" s="27"/>
+      <c r="F29" s="28"/>
+      <c r="G29" s="28"/>
+      <c r="H29" s="27"/>
+      <c r="I29" s="28"/>
+      <c r="J29" s="11"/>
+    </row>
+    <row r="30" spans="1:12" customHeight="1" ht="32.1">
+      <c r="A30" s="29"/>
+      <c r="B30" s="30"/>
+      <c r="C30" s="29"/>
+      <c r="D30" s="30"/>
+      <c r="E30" s="29"/>
+      <c r="F30" s="30"/>
+      <c r="G30" s="30"/>
+      <c r="H30" s="29"/>
+      <c r="I30" s="30"/>
+      <c r="J30" s="11"/>
+    </row>
+    <row r="31" spans="1:12" customHeight="1" ht="32.1">
+      <c r="A31" s="27"/>
+      <c r="B31" s="28"/>
+      <c r="C31" s="27"/>
+      <c r="D31" s="28"/>
+      <c r="E31" s="27"/>
+      <c r="F31" s="28"/>
+      <c r="G31" s="28"/>
+      <c r="H31" s="27"/>
+      <c r="I31" s="28"/>
+      <c r="J31" s="11"/>
+    </row>
+    <row r="32" spans="1:12" customHeight="1" ht="32.1">
+      <c r="A32" s="29"/>
+      <c r="B32" s="30"/>
+      <c r="C32" s="29"/>
+      <c r="D32" s="30"/>
+      <c r="E32" s="29"/>
+      <c r="F32" s="30"/>
+      <c r="G32" s="30"/>
+      <c r="H32" s="29"/>
+      <c r="I32" s="30"/>
+      <c r="J32" s="11"/>
+    </row>
+    <row r="33" spans="1:12" customHeight="1" ht="32.1">
+      <c r="A33" s="27"/>
+      <c r="B33" s="28"/>
+      <c r="C33" s="27"/>
+      <c r="D33" s="28"/>
+      <c r="E33" s="27"/>
+      <c r="F33" s="28"/>
+      <c r="G33" s="28"/>
+      <c r="H33" s="27"/>
+      <c r="I33" s="28"/>
+      <c r="J33" s="11"/>
+    </row>
+    <row r="34" spans="1:12" customHeight="1" ht="32.1">
+      <c r="A34" s="29"/>
+      <c r="B34" s="30"/>
+      <c r="C34" s="29"/>
+      <c r="D34" s="30"/>
+      <c r="E34" s="29"/>
+      <c r="F34" s="30"/>
+      <c r="G34" s="30"/>
+      <c r="H34" s="29"/>
+      <c r="I34" s="30"/>
+      <c r="J34" s="11"/>
+    </row>
+    <row r="35" spans="1:12" customHeight="1" ht="32.1">
+      <c r="A35" s="27"/>
+      <c r="B35" s="28"/>
+      <c r="C35" s="27"/>
+      <c r="D35" s="28"/>
+      <c r="E35" s="27"/>
+      <c r="F35" s="28"/>
+      <c r="G35" s="28"/>
+      <c r="H35" s="27"/>
+      <c r="I35" s="28"/>
+      <c r="J35" s="11"/>
+    </row>
+    <row r="36" spans="1:12" customHeight="1" ht="32.1">
+      <c r="A36" s="29"/>
+      <c r="B36" s="30"/>
+      <c r="C36" s="29"/>
+      <c r="D36" s="30"/>
+      <c r="E36" s="29"/>
+      <c r="F36" s="30"/>
+      <c r="G36" s="30"/>
+      <c r="H36" s="29"/>
+      <c r="I36" s="30"/>
+      <c r="J36" s="11"/>
+    </row>
+    <row r="37" spans="1:12" customHeight="1" ht="32.1">
+      <c r="A37" s="27"/>
+      <c r="B37" s="28"/>
+      <c r="C37" s="27"/>
+      <c r="D37" s="28"/>
+      <c r="E37" s="27"/>
+      <c r="F37" s="28"/>
+      <c r="G37" s="28"/>
+      <c r="H37" s="27"/>
+      <c r="I37" s="28"/>
+      <c r="J37" s="11"/>
+    </row>
+    <row r="38" spans="1:12" customHeight="1" ht="32.1">
+      <c r="A38" s="29"/>
+      <c r="B38" s="30"/>
+      <c r="C38" s="29"/>
+      <c r="D38" s="30"/>
+      <c r="E38" s="29"/>
+      <c r="F38" s="30"/>
+      <c r="G38" s="30"/>
+      <c r="H38" s="29"/>
+      <c r="I38" s="30"/>
+      <c r="J38" s="11"/>
+    </row>
+    <row r="39" spans="1:12" customHeight="1" ht="32.1">
+      <c r="A39" s="27"/>
+      <c r="B39" s="28"/>
+      <c r="C39" s="27"/>
+      <c r="D39" s="28"/>
+      <c r="E39" s="27"/>
+      <c r="F39" s="28"/>
+      <c r="G39" s="28"/>
+      <c r="H39" s="27"/>
+      <c r="I39" s="28"/>
+      <c r="J39" s="11"/>
+    </row>
+    <row r="40" spans="1:12" customHeight="1" ht="32.1">
+      <c r="A40" s="29"/>
+      <c r="B40" s="30"/>
+      <c r="C40" s="29"/>
+      <c r="D40" s="30"/>
+      <c r="E40" s="29"/>
+      <c r="F40" s="30"/>
+      <c r="G40" s="30"/>
+      <c r="H40" s="29"/>
+      <c r="I40" s="30"/>
+      <c r="J40" s="11"/>
+    </row>
+    <row r="41" spans="1:12" customHeight="1" ht="32.1">
+      <c r="A41" s="27"/>
+      <c r="B41" s="28"/>
+      <c r="C41" s="27"/>
+      <c r="D41" s="28"/>
+      <c r="E41" s="27"/>
+      <c r="F41" s="28"/>
+      <c r="G41" s="28"/>
+      <c r="H41" s="27"/>
+      <c r="I41" s="28"/>
+      <c r="J41" s="11"/>
+    </row>
+    <row r="42" spans="1:12" customHeight="1" ht="32.1">
+      <c r="A42" s="29"/>
+      <c r="B42" s="30"/>
+      <c r="C42" s="29"/>
+      <c r="D42" s="30"/>
+      <c r="E42" s="29"/>
+      <c r="F42" s="30"/>
+      <c r="G42" s="30"/>
+      <c r="H42" s="29"/>
+      <c r="I42" s="30"/>
+      <c r="J42" s="11"/>
+    </row>
+    <row r="43" spans="1:12" customHeight="1" ht="32.1">
+      <c r="A43" s="27"/>
+      <c r="B43" s="28"/>
+      <c r="C43" s="27"/>
+      <c r="D43" s="28"/>
+      <c r="E43" s="27"/>
+      <c r="F43" s="28"/>
+      <c r="G43" s="28"/>
+      <c r="H43" s="27"/>
+      <c r="I43" s="28"/>
+      <c r="J43" s="11"/>
+    </row>
+    <row r="44" spans="1:12" customHeight="1" ht="32.1">
+      <c r="A44" s="29"/>
+      <c r="B44" s="30"/>
+      <c r="C44" s="29"/>
+      <c r="D44" s="30"/>
+      <c r="E44" s="29"/>
+      <c r="F44" s="30"/>
+      <c r="G44" s="30"/>
+      <c r="H44" s="29"/>
+      <c r="I44" s="30"/>
+      <c r="J44" s="11"/>
+    </row>
+    <row r="45" spans="1:12" customHeight="1" ht="32.1">
+      <c r="A45" s="27"/>
+      <c r="B45" s="28"/>
+      <c r="C45" s="27"/>
+      <c r="D45" s="28"/>
+      <c r="E45" s="27"/>
+      <c r="F45" s="28"/>
+      <c r="G45" s="28"/>
+      <c r="H45" s="27"/>
+      <c r="I45" s="28"/>
+      <c r="J45" s="11"/>
+    </row>
+    <row r="46" spans="1:12" customHeight="1" ht="32.1">
+      <c r="A46" s="29"/>
+      <c r="B46" s="30"/>
+      <c r="C46" s="29"/>
+      <c r="D46" s="30"/>
+      <c r="E46" s="29"/>
+      <c r="F46" s="30"/>
+      <c r="G46" s="30"/>
+      <c r="H46" s="29"/>
+      <c r="I46" s="30"/>
+      <c r="J46" s="11"/>
+    </row>
+    <row r="47" spans="1:12" customHeight="1" ht="32.1">
+      <c r="A47" s="27"/>
+      <c r="B47" s="28"/>
+      <c r="C47" s="27"/>
+      <c r="D47" s="28"/>
+      <c r="E47" s="27"/>
+      <c r="F47" s="28"/>
+      <c r="G47" s="28"/>
+      <c r="H47" s="27"/>
+      <c r="I47" s="28"/>
+      <c r="J47" s="11"/>
+    </row>
+    <row r="48" spans="1:12" customHeight="1" ht="32.1">
+      <c r="A48" s="29"/>
+      <c r="B48" s="30"/>
+      <c r="C48" s="29"/>
+      <c r="D48" s="30"/>
+      <c r="E48" s="29"/>
+      <c r="F48" s="30"/>
+      <c r="G48" s="30"/>
+      <c r="H48" s="29"/>
+      <c r="I48" s="30"/>
+      <c r="J48" s="11"/>
+    </row>
+  </sheetData>
+  <mergeCells>
+    <mergeCell ref="A48:B48"/>
+    <mergeCell ref="C48:D48"/>
+    <mergeCell ref="E48:G48"/>
+    <mergeCell ref="H48:I48"/>
+    <mergeCell ref="A46:B46"/>
+    <mergeCell ref="C46:D46"/>
+    <mergeCell ref="E46:G46"/>
+    <mergeCell ref="H46:I46"/>
+    <mergeCell ref="A47:B47"/>
+    <mergeCell ref="C47:D47"/>
+    <mergeCell ref="E47:G47"/>
+    <mergeCell ref="H47:I47"/>
+    <mergeCell ref="A44:B44"/>
+    <mergeCell ref="C44:D44"/>
+    <mergeCell ref="E44:G44"/>
+    <mergeCell ref="H44:I44"/>
+    <mergeCell ref="A45:B45"/>
+    <mergeCell ref="C45:D45"/>
+    <mergeCell ref="E45:G45"/>
+    <mergeCell ref="H45:I45"/>
+    <mergeCell ref="A42:B42"/>
+    <mergeCell ref="C42:D42"/>
+    <mergeCell ref="E42:G42"/>
+    <mergeCell ref="H42:I42"/>
+    <mergeCell ref="A43:B43"/>
+    <mergeCell ref="C43:D43"/>
+    <mergeCell ref="E43:G43"/>
+    <mergeCell ref="H43:I43"/>
+    <mergeCell ref="A40:B40"/>
+    <mergeCell ref="C40:D40"/>
+    <mergeCell ref="E40:G40"/>
+    <mergeCell ref="H40:I40"/>
+    <mergeCell ref="A41:B41"/>
+    <mergeCell ref="C41:D41"/>
+    <mergeCell ref="E41:G41"/>
+    <mergeCell ref="H41:I41"/>
+    <mergeCell ref="A38:B38"/>
+    <mergeCell ref="C38:D38"/>
+    <mergeCell ref="E38:G38"/>
+    <mergeCell ref="H38:I38"/>
+    <mergeCell ref="A39:B39"/>
+    <mergeCell ref="C39:D39"/>
+    <mergeCell ref="E39:G39"/>
+    <mergeCell ref="H39:I39"/>
+    <mergeCell ref="A36:B36"/>
+    <mergeCell ref="C36:D36"/>
+    <mergeCell ref="E36:G36"/>
+    <mergeCell ref="H36:I36"/>
+    <mergeCell ref="A37:B37"/>
+    <mergeCell ref="C37:D37"/>
+    <mergeCell ref="E37:G37"/>
+    <mergeCell ref="H37:I37"/>
+    <mergeCell ref="A34:B34"/>
+    <mergeCell ref="C34:D34"/>
+    <mergeCell ref="E34:G34"/>
+    <mergeCell ref="H34:I34"/>
+    <mergeCell ref="A35:B35"/>
+    <mergeCell ref="C35:D35"/>
+    <mergeCell ref="E35:G35"/>
+    <mergeCell ref="H35:I35"/>
+    <mergeCell ref="A32:B32"/>
+    <mergeCell ref="C32:D32"/>
+    <mergeCell ref="E32:G32"/>
+    <mergeCell ref="H32:I32"/>
+    <mergeCell ref="A33:B33"/>
+    <mergeCell ref="C33:D33"/>
+    <mergeCell ref="E33:G33"/>
+    <mergeCell ref="H33:I33"/>
+    <mergeCell ref="A30:B30"/>
+    <mergeCell ref="C30:D30"/>
+    <mergeCell ref="E30:G30"/>
+    <mergeCell ref="H30:I30"/>
+    <mergeCell ref="A31:B31"/>
+    <mergeCell ref="C31:D31"/>
+    <mergeCell ref="E31:G31"/>
+    <mergeCell ref="H31:I31"/>
+    <mergeCell ref="A28:B28"/>
+    <mergeCell ref="C28:D28"/>
+    <mergeCell ref="E28:G28"/>
+    <mergeCell ref="H28:I28"/>
+    <mergeCell ref="A29:B29"/>
+    <mergeCell ref="C29:D29"/>
+    <mergeCell ref="E29:G29"/>
+    <mergeCell ref="H29:I29"/>
+    <mergeCell ref="A26:B26"/>
+    <mergeCell ref="C26:D26"/>
+    <mergeCell ref="E26:G26"/>
+    <mergeCell ref="H26:I26"/>
+    <mergeCell ref="A27:B27"/>
+    <mergeCell ref="C27:D27"/>
+    <mergeCell ref="E27:G27"/>
+    <mergeCell ref="H27:I27"/>
+    <mergeCell ref="A24:B24"/>
+    <mergeCell ref="C24:D24"/>
+    <mergeCell ref="E24:G24"/>
+    <mergeCell ref="H24:I24"/>
+    <mergeCell ref="A25:B25"/>
+    <mergeCell ref="C25:D25"/>
+    <mergeCell ref="E25:G25"/>
+    <mergeCell ref="H25:I25"/>
+    <mergeCell ref="A22:B22"/>
+    <mergeCell ref="C22:D22"/>
+    <mergeCell ref="E22:G22"/>
+    <mergeCell ref="H22:I22"/>
+    <mergeCell ref="A23:B23"/>
+    <mergeCell ref="C23:D23"/>
+    <mergeCell ref="E23:G23"/>
+    <mergeCell ref="H23:I23"/>
+    <mergeCell ref="A20:B20"/>
+    <mergeCell ref="C20:D20"/>
+    <mergeCell ref="E20:G20"/>
+    <mergeCell ref="H20:I20"/>
+    <mergeCell ref="A21:B21"/>
+    <mergeCell ref="C21:D21"/>
+    <mergeCell ref="E21:G21"/>
+    <mergeCell ref="H21:I21"/>
+    <mergeCell ref="A18:B18"/>
+    <mergeCell ref="C18:D18"/>
+    <mergeCell ref="E18:G18"/>
+    <mergeCell ref="H18:I18"/>
+    <mergeCell ref="A19:B19"/>
+    <mergeCell ref="C19:D19"/>
+    <mergeCell ref="E19:G19"/>
+    <mergeCell ref="H19:I19"/>
+    <mergeCell ref="A16:B16"/>
+    <mergeCell ref="C16:D16"/>
+    <mergeCell ref="E16:G16"/>
+    <mergeCell ref="H16:I16"/>
+    <mergeCell ref="A17:B17"/>
+    <mergeCell ref="C17:D17"/>
+    <mergeCell ref="E17:G17"/>
+    <mergeCell ref="H17:I17"/>
+    <mergeCell ref="A14:B14"/>
+    <mergeCell ref="C14:D14"/>
+    <mergeCell ref="E14:G14"/>
+    <mergeCell ref="H14:I14"/>
+    <mergeCell ref="A15:B15"/>
+    <mergeCell ref="C15:D15"/>
+    <mergeCell ref="E15:G15"/>
+    <mergeCell ref="H15:I15"/>
+    <mergeCell ref="A12:B12"/>
+    <mergeCell ref="C12:D12"/>
+    <mergeCell ref="E12:G12"/>
+    <mergeCell ref="H12:I12"/>
+    <mergeCell ref="A13:B13"/>
+    <mergeCell ref="C13:D13"/>
+    <mergeCell ref="E13:G13"/>
+    <mergeCell ref="H13:I13"/>
+    <mergeCell ref="A10:B10"/>
+    <mergeCell ref="C10:D10"/>
+    <mergeCell ref="E10:G10"/>
+    <mergeCell ref="H10:I10"/>
+    <mergeCell ref="A11:B11"/>
+    <mergeCell ref="C11:D11"/>
+    <mergeCell ref="E11:G11"/>
+    <mergeCell ref="H11:I11"/>
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="C4:E4"/>
+    <mergeCell ref="F4:I4"/>
+    <mergeCell ref="A9:B9"/>
+    <mergeCell ref="C9:D9"/>
+    <mergeCell ref="E9:G9"/>
+    <mergeCell ref="H9:I9"/>
+    <mergeCell ref="A8:B8"/>
+    <mergeCell ref="C8:D8"/>
+    <mergeCell ref="D2:E2"/>
+    <mergeCell ref="E8:G8"/>
+    <mergeCell ref="H8:I8"/>
+    <mergeCell ref="F5:I5"/>
+    <mergeCell ref="A5:B5"/>
+    <mergeCell ref="C5:E5"/>
+    <mergeCell ref="B3:D3"/>
+  </mergeCells>
+  <printOptions gridLines="false" gridLinesSet="true"/>
+  <pageMargins left="0.70866141732283" right="0.51181102362205" top="0.74803149606299" bottom="0.74803149606299" header="0.31496062992126" footer="0.31496062992126"/>
+  <pageSetup paperSize="9" orientation="portrait" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" r:id="rId1ps"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Skladová karta: jeden list, duplex jako papír (zlom po ř. 25).
Deník 17+22 řádků na jednom listu dle etalonu; bez fit-to-page, strana 2 od hlavičky deníku (ř. 26).

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/deploy/excel/skladova-karta.template.xlsx
+++ b/deploy/excel/skladova-karta.template.xlsx
@@ -7,8 +7,7 @@
     <workbookView activeTab="0" autoFilterDateGrouping="true" firstSheet="0" minimized="false" showHorizontalScroll="true" showSheetTabs="true" showVerticalScroll="true" tabRatio="600" visibility="visible"/>
   </bookViews>
   <sheets>
-    <sheet name="Strana 1" sheetId="1" r:id="rId4"/>
-    <sheet name="Strana 2" sheetId="2" r:id="rId5"/>
+    <sheet name="Skladová karta" sheetId="1" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="999999" calcMode="auto" calcCompleted="1" fullCalcOnLoad="0" forceFullCalc="0"/>
@@ -16,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="12">
   <si>
     <t>SKLADOVÁ KARTA - OPTIKA</t>
   </si>
@@ -27,45 +26,10 @@
     <t>POČET VLÁKEN:</t>
   </si>
   <si>
-    <t>4 vl</t>
-  </si>
-  <si>
     <t>ŠARŽE:</t>
   </si>
   <si>
-    <t>450-020858</t>
-  </si>
-  <si>
     <t>TYP OK:</t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">MLT  DROP  </t>
-    </r>
-    <r>
-      <rPr>
-        <rFont val="Calibri"/>
-        <b val="false"/>
-        <i val="false"/>
-        <strike val="false"/>
-        <color rgb="FF000000"/>
-        <sz val="11"/>
-        <u val="single"/>
-      </rPr>
-      <t xml:space="preserve">BLOWN</t>
-    </r>
-    <r>
-      <rPr>
-        <rFont val="Calibri"/>
-        <b val="false"/>
-        <i val="false"/>
-        <strike val="false"/>
-        <color rgb="FF000000"/>
-        <sz val="11"/>
-        <u val="none"/>
-      </rPr>
-      <t xml:space="preserve">  FLAT</t>
-    </r>
   </si>
   <si>
     <t>CELKOVÁ METRÁŽ</t>
@@ -757,71 +721,57 @@
       </c>
       <c r="B2" s="3"/>
       <c r="C2" s="3"/>
-      <c r="D2" s="12">
-        <v>46167</v>
-      </c>
+      <c r="D2" s="12"/>
       <c r="E2" s="13"/>
       <c r="F2" s="31" t="s">
         <v>2</v>
       </c>
       <c r="G2" s="5"/>
       <c r="H2" s="3"/>
-      <c r="I2" s="9" t="s">
-        <v>3</v>
-      </c>
+      <c r="I2" s="9"/>
       <c r="J2" s="8"/>
       <c r="K2" s="8"/>
     </row>
     <row r="3" spans="1:12" customHeight="1" ht="33.75">
       <c r="A3" s="32" t="s">
-        <v>4</v>
-      </c>
-      <c r="B3" s="22" t="s">
-        <v>5</v>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="B3" s="22"/>
       <c r="C3" s="22"/>
       <c r="D3" s="22"/>
       <c r="E3" s="7"/>
       <c r="F3" s="35" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="G3" s="5"/>
-      <c r="H3" s="6" t="s">
-        <v>7</v>
-      </c>
+      <c r="H3" s="6"/>
       <c r="I3" s="4"/>
       <c r="J3" s="11"/>
     </row>
     <row r="4" spans="1:12" customHeight="1" ht="26.25">
       <c r="A4" s="33" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="B4" s="34"/>
       <c r="C4" s="33" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="D4" s="36"/>
       <c r="E4" s="34"/>
       <c r="F4" s="24" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="G4" s="25"/>
       <c r="H4" s="25"/>
       <c r="I4" s="26"/>
     </row>
     <row r="5" spans="1:12" customHeight="1" ht="35.25">
-      <c r="A5" s="17">
-        <v>2100</v>
-      </c>
+      <c r="A5" s="17"/>
       <c r="B5" s="18"/>
-      <c r="C5" s="19">
-        <v>4500</v>
-      </c>
+      <c r="C5" s="19"/>
       <c r="D5" s="20"/>
       <c r="E5" s="21"/>
-      <c r="F5" s="14">
-        <v>2</v>
-      </c>
+      <c r="F5" s="14"/>
       <c r="G5" s="15"/>
       <c r="H5" s="15"/>
       <c r="I5" s="16"/>
@@ -842,20 +792,20 @@
     </row>
     <row r="8" spans="1:12" customHeight="1" ht="32.1">
       <c r="A8" s="39" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="B8" s="40"/>
       <c r="C8" s="37" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="D8" s="38"/>
       <c r="E8" s="37" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="F8" s="38"/>
       <c r="G8" s="38"/>
       <c r="H8" s="37" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="I8" s="38"/>
       <c r="J8" s="11"/>
@@ -1065,14 +1015,22 @@
       <c r="J25" s="11"/>
     </row>
     <row r="26" spans="1:12" customHeight="1" ht="32.1">
-      <c r="A26" s="37"/>
+      <c r="A26" s="37" t="s">
+        <v>8</v>
+      </c>
       <c r="B26" s="38"/>
-      <c r="C26" s="37"/>
+      <c r="C26" s="37" t="s">
+        <v>9</v>
+      </c>
       <c r="D26" s="38"/>
-      <c r="E26" s="37"/>
+      <c r="E26" s="37" t="s">
+        <v>10</v>
+      </c>
       <c r="F26" s="38"/>
       <c r="G26" s="38"/>
-      <c r="H26" s="37"/>
+      <c r="H26" s="37" t="s">
+        <v>11</v>
+      </c>
       <c r="I26" s="38"/>
       <c r="J26" s="11"/>
     </row>
@@ -1518,812 +1476,9 @@
   </mergeCells>
   <printOptions gridLines="false" gridLinesSet="true"/>
   <pageMargins left="0.70866141732283" right="0.51181102362205" top="0.74803149606299" bottom="0.74803149606299" header="0.31496062992126" footer="0.31496062992126"/>
-  <pageSetup paperSize="9" orientation="portrait" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" r:id="rId1ps"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xml:space="preserve" mc:Ignorable="x14ac">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-  </sheetPr>
-  <dimension ref="A1:L48"/>
-  <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
-  <cols>
-    <col min="1" max="1" width="9.28515625" customWidth="true" style="0"/>
-    <col min="2" max="2" width="10.28515625" customWidth="true" style="0"/>
-    <col min="4" max="4" width="13" customWidth="true" style="0"/>
-    <col min="5" max="5" width="7.28515625" customWidth="true" style="0"/>
-    <col min="6" max="6" width="9.28515625" customWidth="true" style="0"/>
-    <col min="7" max="7" width="6.7109375" customWidth="true" style="0"/>
-    <col min="8" max="8" width="6.85546875" customWidth="true" style="0"/>
-    <col min="9" max="9" width="16.42578125" customWidth="true" style="0"/>
-    <col min="10" max="10" width="1" customWidth="true" style="0"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:12" customHeight="1" ht="28.5">
-      <c r="A1" s="23" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="23"/>
-      <c r="C1" s="23"/>
-      <c r="D1" s="23"/>
-      <c r="E1" s="23"/>
-      <c r="F1" s="23"/>
-      <c r="G1" s="23"/>
-      <c r="H1" s="23"/>
-      <c r="I1" s="23"/>
-      <c r="J1" s="1"/>
-      <c r="K1" s="1"/>
-      <c r="L1" s="1"/>
-    </row>
-    <row r="2" spans="1:12" customHeight="1" ht="33">
-      <c r="A2" s="31" t="s">
-        <v>1</v>
-      </c>
-      <c r="B2" s="3"/>
-      <c r="C2" s="3"/>
-      <c r="D2" s="12">
-        <v>46167</v>
-      </c>
-      <c r="E2" s="13"/>
-      <c r="F2" s="31" t="s">
-        <v>2</v>
-      </c>
-      <c r="G2" s="5"/>
-      <c r="H2" s="3"/>
-      <c r="I2" s="9" t="s">
-        <v>3</v>
-      </c>
-      <c r="J2" s="8"/>
-      <c r="K2" s="8"/>
-    </row>
-    <row r="3" spans="1:12" customHeight="1" ht="33.75">
-      <c r="A3" s="32" t="s">
-        <v>4</v>
-      </c>
-      <c r="B3" s="22" t="s">
-        <v>5</v>
-      </c>
-      <c r="C3" s="22"/>
-      <c r="D3" s="22"/>
-      <c r="E3" s="7"/>
-      <c r="F3" s="35" t="s">
-        <v>6</v>
-      </c>
-      <c r="G3" s="5"/>
-      <c r="H3" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="I3" s="4"/>
-      <c r="J3" s="11"/>
-    </row>
-    <row r="4" spans="1:12" customHeight="1" ht="26.25">
-      <c r="A4" s="33" t="s">
-        <v>8</v>
-      </c>
-      <c r="B4" s="34"/>
-      <c r="C4" s="33" t="s">
-        <v>9</v>
-      </c>
-      <c r="D4" s="36"/>
-      <c r="E4" s="34"/>
-      <c r="F4" s="24" t="s">
-        <v>10</v>
-      </c>
-      <c r="G4" s="25"/>
-      <c r="H4" s="25"/>
-      <c r="I4" s="26"/>
-    </row>
-    <row r="5" spans="1:12" customHeight="1" ht="35.25">
-      <c r="A5" s="17">
-        <v>2100</v>
-      </c>
-      <c r="B5" s="18"/>
-      <c r="C5" s="19">
-        <v>4500</v>
-      </c>
-      <c r="D5" s="20"/>
-      <c r="E5" s="21"/>
-      <c r="F5" s="14">
-        <v>2</v>
-      </c>
-      <c r="G5" s="15"/>
-      <c r="H5" s="15"/>
-      <c r="I5" s="16"/>
-    </row>
-    <row r="6" spans="1:12" customHeight="1" ht="9">
-      <c r="A6" s="10"/>
-      <c r="B6" s="10"/>
-      <c r="C6" s="10"/>
-      <c r="D6" s="10"/>
-      <c r="E6" s="10"/>
-      <c r="F6" s="10"/>
-      <c r="G6" s="10"/>
-      <c r="H6" s="10"/>
-      <c r="I6" s="10"/>
-    </row>
-    <row r="7" spans="1:12" customHeight="1" ht="12">
-      <c r="I7" s="2"/>
-    </row>
-    <row r="8" spans="1:12" customHeight="1" ht="32.1">
-      <c r="A8" s="39" t="s">
-        <v>11</v>
-      </c>
-      <c r="B8" s="40"/>
-      <c r="C8" s="37" t="s">
-        <v>12</v>
-      </c>
-      <c r="D8" s="38"/>
-      <c r="E8" s="37" t="s">
-        <v>13</v>
-      </c>
-      <c r="F8" s="38"/>
-      <c r="G8" s="38"/>
-      <c r="H8" s="37" t="s">
-        <v>14</v>
-      </c>
-      <c r="I8" s="38"/>
-      <c r="J8" s="11"/>
-    </row>
-    <row r="9" spans="1:12" customHeight="1" ht="32.1">
-      <c r="A9" s="27"/>
-      <c r="B9" s="28"/>
-      <c r="C9" s="27"/>
-      <c r="D9" s="28"/>
-      <c r="E9" s="27"/>
-      <c r="F9" s="28"/>
-      <c r="G9" s="28"/>
-      <c r="H9" s="27"/>
-      <c r="I9" s="28"/>
-      <c r="J9" s="11"/>
-    </row>
-    <row r="10" spans="1:12" customHeight="1" ht="32.1">
-      <c r="A10" s="29"/>
-      <c r="B10" s="30"/>
-      <c r="C10" s="29"/>
-      <c r="D10" s="30"/>
-      <c r="E10" s="29"/>
-      <c r="F10" s="30"/>
-      <c r="G10" s="30"/>
-      <c r="H10" s="29"/>
-      <c r="I10" s="30"/>
-      <c r="J10" s="11"/>
-    </row>
-    <row r="11" spans="1:12" customHeight="1" ht="32.1">
-      <c r="A11" s="27"/>
-      <c r="B11" s="28"/>
-      <c r="C11" s="27"/>
-      <c r="D11" s="28"/>
-      <c r="E11" s="27"/>
-      <c r="F11" s="28"/>
-      <c r="G11" s="28"/>
-      <c r="H11" s="27"/>
-      <c r="I11" s="28"/>
-      <c r="J11" s="11"/>
-    </row>
-    <row r="12" spans="1:12" customHeight="1" ht="32.1">
-      <c r="A12" s="29"/>
-      <c r="B12" s="30"/>
-      <c r="C12" s="29"/>
-      <c r="D12" s="30"/>
-      <c r="E12" s="29"/>
-      <c r="F12" s="30"/>
-      <c r="G12" s="30"/>
-      <c r="H12" s="29"/>
-      <c r="I12" s="30"/>
-      <c r="J12" s="11"/>
-    </row>
-    <row r="13" spans="1:12" customHeight="1" ht="32.1">
-      <c r="A13" s="27"/>
-      <c r="B13" s="28"/>
-      <c r="C13" s="27"/>
-      <c r="D13" s="28"/>
-      <c r="E13" s="27"/>
-      <c r="F13" s="28"/>
-      <c r="G13" s="28"/>
-      <c r="H13" s="27"/>
-      <c r="I13" s="28"/>
-      <c r="J13" s="11"/>
-    </row>
-    <row r="14" spans="1:12" customHeight="1" ht="32.1">
-      <c r="A14" s="29"/>
-      <c r="B14" s="30"/>
-      <c r="C14" s="29"/>
-      <c r="D14" s="30"/>
-      <c r="E14" s="29"/>
-      <c r="F14" s="30"/>
-      <c r="G14" s="30"/>
-      <c r="H14" s="29"/>
-      <c r="I14" s="30"/>
-      <c r="J14" s="11"/>
-    </row>
-    <row r="15" spans="1:12" customHeight="1" ht="32.1">
-      <c r="A15" s="27"/>
-      <c r="B15" s="28"/>
-      <c r="C15" s="27"/>
-      <c r="D15" s="28"/>
-      <c r="E15" s="27"/>
-      <c r="F15" s="28"/>
-      <c r="G15" s="28"/>
-      <c r="H15" s="27"/>
-      <c r="I15" s="28"/>
-      <c r="J15" s="11"/>
-    </row>
-    <row r="16" spans="1:12" customHeight="1" ht="32.1">
-      <c r="A16" s="29"/>
-      <c r="B16" s="30"/>
-      <c r="C16" s="29"/>
-      <c r="D16" s="30"/>
-      <c r="E16" s="29"/>
-      <c r="F16" s="30"/>
-      <c r="G16" s="30"/>
-      <c r="H16" s="29"/>
-      <c r="I16" s="30"/>
-      <c r="J16" s="11"/>
-    </row>
-    <row r="17" spans="1:12" customHeight="1" ht="32.1">
-      <c r="A17" s="27"/>
-      <c r="B17" s="28"/>
-      <c r="C17" s="27"/>
-      <c r="D17" s="28"/>
-      <c r="E17" s="27"/>
-      <c r="F17" s="28"/>
-      <c r="G17" s="28"/>
-      <c r="H17" s="27"/>
-      <c r="I17" s="28"/>
-      <c r="J17" s="11"/>
-    </row>
-    <row r="18" spans="1:12" customHeight="1" ht="32.1">
-      <c r="A18" s="29"/>
-      <c r="B18" s="30"/>
-      <c r="C18" s="29"/>
-      <c r="D18" s="30"/>
-      <c r="E18" s="29"/>
-      <c r="F18" s="30"/>
-      <c r="G18" s="30"/>
-      <c r="H18" s="29"/>
-      <c r="I18" s="30"/>
-      <c r="J18" s="11"/>
-    </row>
-    <row r="19" spans="1:12" customHeight="1" ht="32.1">
-      <c r="A19" s="27"/>
-      <c r="B19" s="28"/>
-      <c r="C19" s="27"/>
-      <c r="D19" s="28"/>
-      <c r="E19" s="27"/>
-      <c r="F19" s="28"/>
-      <c r="G19" s="28"/>
-      <c r="H19" s="27"/>
-      <c r="I19" s="28"/>
-      <c r="J19" s="11"/>
-    </row>
-    <row r="20" spans="1:12" customHeight="1" ht="32.1">
-      <c r="A20" s="29"/>
-      <c r="B20" s="30"/>
-      <c r="C20" s="29"/>
-      <c r="D20" s="30"/>
-      <c r="E20" s="29"/>
-      <c r="F20" s="30"/>
-      <c r="G20" s="30"/>
-      <c r="H20" s="29"/>
-      <c r="I20" s="30"/>
-      <c r="J20" s="11"/>
-    </row>
-    <row r="21" spans="1:12" customHeight="1" ht="32.1">
-      <c r="A21" s="27"/>
-      <c r="B21" s="28"/>
-      <c r="C21" s="27"/>
-      <c r="D21" s="28"/>
-      <c r="E21" s="27"/>
-      <c r="F21" s="28"/>
-      <c r="G21" s="28"/>
-      <c r="H21" s="27"/>
-      <c r="I21" s="28"/>
-      <c r="J21" s="11"/>
-    </row>
-    <row r="22" spans="1:12" customHeight="1" ht="32.1">
-      <c r="A22" s="29"/>
-      <c r="B22" s="30"/>
-      <c r="C22" s="29"/>
-      <c r="D22" s="30"/>
-      <c r="E22" s="29"/>
-      <c r="F22" s="30"/>
-      <c r="G22" s="30"/>
-      <c r="H22" s="29"/>
-      <c r="I22" s="30"/>
-      <c r="J22" s="11"/>
-    </row>
-    <row r="23" spans="1:12" customHeight="1" ht="32.1">
-      <c r="A23" s="27"/>
-      <c r="B23" s="28"/>
-      <c r="C23" s="27"/>
-      <c r="D23" s="28"/>
-      <c r="E23" s="27"/>
-      <c r="F23" s="28"/>
-      <c r="G23" s="28"/>
-      <c r="H23" s="27"/>
-      <c r="I23" s="28"/>
-      <c r="J23" s="11"/>
-    </row>
-    <row r="24" spans="1:12" customHeight="1" ht="32.1">
-      <c r="A24" s="29"/>
-      <c r="B24" s="30"/>
-      <c r="C24" s="29"/>
-      <c r="D24" s="30"/>
-      <c r="E24" s="29"/>
-      <c r="F24" s="30"/>
-      <c r="G24" s="30"/>
-      <c r="H24" s="29"/>
-      <c r="I24" s="30"/>
-      <c r="J24" s="11"/>
-    </row>
-    <row r="25" spans="1:12" customHeight="1" ht="32.1">
-      <c r="A25" s="27"/>
-      <c r="B25" s="28"/>
-      <c r="C25" s="27"/>
-      <c r="D25" s="28"/>
-      <c r="E25" s="27"/>
-      <c r="F25" s="28"/>
-      <c r="G25" s="28"/>
-      <c r="H25" s="27"/>
-      <c r="I25" s="28"/>
-      <c r="J25" s="11"/>
-    </row>
-    <row r="26" spans="1:12" customHeight="1" ht="32.1">
-      <c r="A26" s="37"/>
-      <c r="B26" s="38"/>
-      <c r="C26" s="37"/>
-      <c r="D26" s="38"/>
-      <c r="E26" s="37"/>
-      <c r="F26" s="38"/>
-      <c r="G26" s="38"/>
-      <c r="H26" s="37"/>
-      <c r="I26" s="38"/>
-      <c r="J26" s="11"/>
-    </row>
-    <row r="27" spans="1:12" customHeight="1" ht="32.1">
-      <c r="A27" s="27"/>
-      <c r="B27" s="28"/>
-      <c r="C27" s="27"/>
-      <c r="D27" s="28"/>
-      <c r="E27" s="27"/>
-      <c r="F27" s="28"/>
-      <c r="G27" s="28"/>
-      <c r="H27" s="27"/>
-      <c r="I27" s="28"/>
-      <c r="J27" s="11"/>
-    </row>
-    <row r="28" spans="1:12" customHeight="1" ht="32.1">
-      <c r="A28" s="29"/>
-      <c r="B28" s="30"/>
-      <c r="C28" s="29"/>
-      <c r="D28" s="30"/>
-      <c r="E28" s="29"/>
-      <c r="F28" s="30"/>
-      <c r="G28" s="30"/>
-      <c r="H28" s="29"/>
-      <c r="I28" s="30"/>
-      <c r="J28" s="11"/>
-    </row>
-    <row r="29" spans="1:12" customHeight="1" ht="32.1">
-      <c r="A29" s="27"/>
-      <c r="B29" s="28"/>
-      <c r="C29" s="27"/>
-      <c r="D29" s="28"/>
-      <c r="E29" s="27"/>
-      <c r="F29" s="28"/>
-      <c r="G29" s="28"/>
-      <c r="H29" s="27"/>
-      <c r="I29" s="28"/>
-      <c r="J29" s="11"/>
-    </row>
-    <row r="30" spans="1:12" customHeight="1" ht="32.1">
-      <c r="A30" s="29"/>
-      <c r="B30" s="30"/>
-      <c r="C30" s="29"/>
-      <c r="D30" s="30"/>
-      <c r="E30" s="29"/>
-      <c r="F30" s="30"/>
-      <c r="G30" s="30"/>
-      <c r="H30" s="29"/>
-      <c r="I30" s="30"/>
-      <c r="J30" s="11"/>
-    </row>
-    <row r="31" spans="1:12" customHeight="1" ht="32.1">
-      <c r="A31" s="27"/>
-      <c r="B31" s="28"/>
-      <c r="C31" s="27"/>
-      <c r="D31" s="28"/>
-      <c r="E31" s="27"/>
-      <c r="F31" s="28"/>
-      <c r="G31" s="28"/>
-      <c r="H31" s="27"/>
-      <c r="I31" s="28"/>
-      <c r="J31" s="11"/>
-    </row>
-    <row r="32" spans="1:12" customHeight="1" ht="32.1">
-      <c r="A32" s="29"/>
-      <c r="B32" s="30"/>
-      <c r="C32" s="29"/>
-      <c r="D32" s="30"/>
-      <c r="E32" s="29"/>
-      <c r="F32" s="30"/>
-      <c r="G32" s="30"/>
-      <c r="H32" s="29"/>
-      <c r="I32" s="30"/>
-      <c r="J32" s="11"/>
-    </row>
-    <row r="33" spans="1:12" customHeight="1" ht="32.1">
-      <c r="A33" s="27"/>
-      <c r="B33" s="28"/>
-      <c r="C33" s="27"/>
-      <c r="D33" s="28"/>
-      <c r="E33" s="27"/>
-      <c r="F33" s="28"/>
-      <c r="G33" s="28"/>
-      <c r="H33" s="27"/>
-      <c r="I33" s="28"/>
-      <c r="J33" s="11"/>
-    </row>
-    <row r="34" spans="1:12" customHeight="1" ht="32.1">
-      <c r="A34" s="29"/>
-      <c r="B34" s="30"/>
-      <c r="C34" s="29"/>
-      <c r="D34" s="30"/>
-      <c r="E34" s="29"/>
-      <c r="F34" s="30"/>
-      <c r="G34" s="30"/>
-      <c r="H34" s="29"/>
-      <c r="I34" s="30"/>
-      <c r="J34" s="11"/>
-    </row>
-    <row r="35" spans="1:12" customHeight="1" ht="32.1">
-      <c r="A35" s="27"/>
-      <c r="B35" s="28"/>
-      <c r="C35" s="27"/>
-      <c r="D35" s="28"/>
-      <c r="E35" s="27"/>
-      <c r="F35" s="28"/>
-      <c r="G35" s="28"/>
-      <c r="H35" s="27"/>
-      <c r="I35" s="28"/>
-      <c r="J35" s="11"/>
-    </row>
-    <row r="36" spans="1:12" customHeight="1" ht="32.1">
-      <c r="A36" s="29"/>
-      <c r="B36" s="30"/>
-      <c r="C36" s="29"/>
-      <c r="D36" s="30"/>
-      <c r="E36" s="29"/>
-      <c r="F36" s="30"/>
-      <c r="G36" s="30"/>
-      <c r="H36" s="29"/>
-      <c r="I36" s="30"/>
-      <c r="J36" s="11"/>
-    </row>
-    <row r="37" spans="1:12" customHeight="1" ht="32.1">
-      <c r="A37" s="27"/>
-      <c r="B37" s="28"/>
-      <c r="C37" s="27"/>
-      <c r="D37" s="28"/>
-      <c r="E37" s="27"/>
-      <c r="F37" s="28"/>
-      <c r="G37" s="28"/>
-      <c r="H37" s="27"/>
-      <c r="I37" s="28"/>
-      <c r="J37" s="11"/>
-    </row>
-    <row r="38" spans="1:12" customHeight="1" ht="32.1">
-      <c r="A38" s="29"/>
-      <c r="B38" s="30"/>
-      <c r="C38" s="29"/>
-      <c r="D38" s="30"/>
-      <c r="E38" s="29"/>
-      <c r="F38" s="30"/>
-      <c r="G38" s="30"/>
-      <c r="H38" s="29"/>
-      <c r="I38" s="30"/>
-      <c r="J38" s="11"/>
-    </row>
-    <row r="39" spans="1:12" customHeight="1" ht="32.1">
-      <c r="A39" s="27"/>
-      <c r="B39" s="28"/>
-      <c r="C39" s="27"/>
-      <c r="D39" s="28"/>
-      <c r="E39" s="27"/>
-      <c r="F39" s="28"/>
-      <c r="G39" s="28"/>
-      <c r="H39" s="27"/>
-      <c r="I39" s="28"/>
-      <c r="J39" s="11"/>
-    </row>
-    <row r="40" spans="1:12" customHeight="1" ht="32.1">
-      <c r="A40" s="29"/>
-      <c r="B40" s="30"/>
-      <c r="C40" s="29"/>
-      <c r="D40" s="30"/>
-      <c r="E40" s="29"/>
-      <c r="F40" s="30"/>
-      <c r="G40" s="30"/>
-      <c r="H40" s="29"/>
-      <c r="I40" s="30"/>
-      <c r="J40" s="11"/>
-    </row>
-    <row r="41" spans="1:12" customHeight="1" ht="32.1">
-      <c r="A41" s="27"/>
-      <c r="B41" s="28"/>
-      <c r="C41" s="27"/>
-      <c r="D41" s="28"/>
-      <c r="E41" s="27"/>
-      <c r="F41" s="28"/>
-      <c r="G41" s="28"/>
-      <c r="H41" s="27"/>
-      <c r="I41" s="28"/>
-      <c r="J41" s="11"/>
-    </row>
-    <row r="42" spans="1:12" customHeight="1" ht="32.1">
-      <c r="A42" s="29"/>
-      <c r="B42" s="30"/>
-      <c r="C42" s="29"/>
-      <c r="D42" s="30"/>
-      <c r="E42" s="29"/>
-      <c r="F42" s="30"/>
-      <c r="G42" s="30"/>
-      <c r="H42" s="29"/>
-      <c r="I42" s="30"/>
-      <c r="J42" s="11"/>
-    </row>
-    <row r="43" spans="1:12" customHeight="1" ht="32.1">
-      <c r="A43" s="27"/>
-      <c r="B43" s="28"/>
-      <c r="C43" s="27"/>
-      <c r="D43" s="28"/>
-      <c r="E43" s="27"/>
-      <c r="F43" s="28"/>
-      <c r="G43" s="28"/>
-      <c r="H43" s="27"/>
-      <c r="I43" s="28"/>
-      <c r="J43" s="11"/>
-    </row>
-    <row r="44" spans="1:12" customHeight="1" ht="32.1">
-      <c r="A44" s="29"/>
-      <c r="B44" s="30"/>
-      <c r="C44" s="29"/>
-      <c r="D44" s="30"/>
-      <c r="E44" s="29"/>
-      <c r="F44" s="30"/>
-      <c r="G44" s="30"/>
-      <c r="H44" s="29"/>
-      <c r="I44" s="30"/>
-      <c r="J44" s="11"/>
-    </row>
-    <row r="45" spans="1:12" customHeight="1" ht="32.1">
-      <c r="A45" s="27"/>
-      <c r="B45" s="28"/>
-      <c r="C45" s="27"/>
-      <c r="D45" s="28"/>
-      <c r="E45" s="27"/>
-      <c r="F45" s="28"/>
-      <c r="G45" s="28"/>
-      <c r="H45" s="27"/>
-      <c r="I45" s="28"/>
-      <c r="J45" s="11"/>
-    </row>
-    <row r="46" spans="1:12" customHeight="1" ht="32.1">
-      <c r="A46" s="29"/>
-      <c r="B46" s="30"/>
-      <c r="C46" s="29"/>
-      <c r="D46" s="30"/>
-      <c r="E46" s="29"/>
-      <c r="F46" s="30"/>
-      <c r="G46" s="30"/>
-      <c r="H46" s="29"/>
-      <c r="I46" s="30"/>
-      <c r="J46" s="11"/>
-    </row>
-    <row r="47" spans="1:12" customHeight="1" ht="32.1">
-      <c r="A47" s="27"/>
-      <c r="B47" s="28"/>
-      <c r="C47" s="27"/>
-      <c r="D47" s="28"/>
-      <c r="E47" s="27"/>
-      <c r="F47" s="28"/>
-      <c r="G47" s="28"/>
-      <c r="H47" s="27"/>
-      <c r="I47" s="28"/>
-      <c r="J47" s="11"/>
-    </row>
-    <row r="48" spans="1:12" customHeight="1" ht="32.1">
-      <c r="A48" s="29"/>
-      <c r="B48" s="30"/>
-      <c r="C48" s="29"/>
-      <c r="D48" s="30"/>
-      <c r="E48" s="29"/>
-      <c r="F48" s="30"/>
-      <c r="G48" s="30"/>
-      <c r="H48" s="29"/>
-      <c r="I48" s="30"/>
-      <c r="J48" s="11"/>
-    </row>
-  </sheetData>
-  <mergeCells>
-    <mergeCell ref="A48:B48"/>
-    <mergeCell ref="C48:D48"/>
-    <mergeCell ref="E48:G48"/>
-    <mergeCell ref="H48:I48"/>
-    <mergeCell ref="A46:B46"/>
-    <mergeCell ref="C46:D46"/>
-    <mergeCell ref="E46:G46"/>
-    <mergeCell ref="H46:I46"/>
-    <mergeCell ref="A47:B47"/>
-    <mergeCell ref="C47:D47"/>
-    <mergeCell ref="E47:G47"/>
-    <mergeCell ref="H47:I47"/>
-    <mergeCell ref="A44:B44"/>
-    <mergeCell ref="C44:D44"/>
-    <mergeCell ref="E44:G44"/>
-    <mergeCell ref="H44:I44"/>
-    <mergeCell ref="A45:B45"/>
-    <mergeCell ref="C45:D45"/>
-    <mergeCell ref="E45:G45"/>
-    <mergeCell ref="H45:I45"/>
-    <mergeCell ref="A42:B42"/>
-    <mergeCell ref="C42:D42"/>
-    <mergeCell ref="E42:G42"/>
-    <mergeCell ref="H42:I42"/>
-    <mergeCell ref="A43:B43"/>
-    <mergeCell ref="C43:D43"/>
-    <mergeCell ref="E43:G43"/>
-    <mergeCell ref="H43:I43"/>
-    <mergeCell ref="A40:B40"/>
-    <mergeCell ref="C40:D40"/>
-    <mergeCell ref="E40:G40"/>
-    <mergeCell ref="H40:I40"/>
-    <mergeCell ref="A41:B41"/>
-    <mergeCell ref="C41:D41"/>
-    <mergeCell ref="E41:G41"/>
-    <mergeCell ref="H41:I41"/>
-    <mergeCell ref="A38:B38"/>
-    <mergeCell ref="C38:D38"/>
-    <mergeCell ref="E38:G38"/>
-    <mergeCell ref="H38:I38"/>
-    <mergeCell ref="A39:B39"/>
-    <mergeCell ref="C39:D39"/>
-    <mergeCell ref="E39:G39"/>
-    <mergeCell ref="H39:I39"/>
-    <mergeCell ref="A36:B36"/>
-    <mergeCell ref="C36:D36"/>
-    <mergeCell ref="E36:G36"/>
-    <mergeCell ref="H36:I36"/>
-    <mergeCell ref="A37:B37"/>
-    <mergeCell ref="C37:D37"/>
-    <mergeCell ref="E37:G37"/>
-    <mergeCell ref="H37:I37"/>
-    <mergeCell ref="A34:B34"/>
-    <mergeCell ref="C34:D34"/>
-    <mergeCell ref="E34:G34"/>
-    <mergeCell ref="H34:I34"/>
-    <mergeCell ref="A35:B35"/>
-    <mergeCell ref="C35:D35"/>
-    <mergeCell ref="E35:G35"/>
-    <mergeCell ref="H35:I35"/>
-    <mergeCell ref="A32:B32"/>
-    <mergeCell ref="C32:D32"/>
-    <mergeCell ref="E32:G32"/>
-    <mergeCell ref="H32:I32"/>
-    <mergeCell ref="A33:B33"/>
-    <mergeCell ref="C33:D33"/>
-    <mergeCell ref="E33:G33"/>
-    <mergeCell ref="H33:I33"/>
-    <mergeCell ref="A30:B30"/>
-    <mergeCell ref="C30:D30"/>
-    <mergeCell ref="E30:G30"/>
-    <mergeCell ref="H30:I30"/>
-    <mergeCell ref="A31:B31"/>
-    <mergeCell ref="C31:D31"/>
-    <mergeCell ref="E31:G31"/>
-    <mergeCell ref="H31:I31"/>
-    <mergeCell ref="A28:B28"/>
-    <mergeCell ref="C28:D28"/>
-    <mergeCell ref="E28:G28"/>
-    <mergeCell ref="H28:I28"/>
-    <mergeCell ref="A29:B29"/>
-    <mergeCell ref="C29:D29"/>
-    <mergeCell ref="E29:G29"/>
-    <mergeCell ref="H29:I29"/>
-    <mergeCell ref="A26:B26"/>
-    <mergeCell ref="C26:D26"/>
-    <mergeCell ref="E26:G26"/>
-    <mergeCell ref="H26:I26"/>
-    <mergeCell ref="A27:B27"/>
-    <mergeCell ref="C27:D27"/>
-    <mergeCell ref="E27:G27"/>
-    <mergeCell ref="H27:I27"/>
-    <mergeCell ref="A24:B24"/>
-    <mergeCell ref="C24:D24"/>
-    <mergeCell ref="E24:G24"/>
-    <mergeCell ref="H24:I24"/>
-    <mergeCell ref="A25:B25"/>
-    <mergeCell ref="C25:D25"/>
-    <mergeCell ref="E25:G25"/>
-    <mergeCell ref="H25:I25"/>
-    <mergeCell ref="A22:B22"/>
-    <mergeCell ref="C22:D22"/>
-    <mergeCell ref="E22:G22"/>
-    <mergeCell ref="H22:I22"/>
-    <mergeCell ref="A23:B23"/>
-    <mergeCell ref="C23:D23"/>
-    <mergeCell ref="E23:G23"/>
-    <mergeCell ref="H23:I23"/>
-    <mergeCell ref="A20:B20"/>
-    <mergeCell ref="C20:D20"/>
-    <mergeCell ref="E20:G20"/>
-    <mergeCell ref="H20:I20"/>
-    <mergeCell ref="A21:B21"/>
-    <mergeCell ref="C21:D21"/>
-    <mergeCell ref="E21:G21"/>
-    <mergeCell ref="H21:I21"/>
-    <mergeCell ref="A18:B18"/>
-    <mergeCell ref="C18:D18"/>
-    <mergeCell ref="E18:G18"/>
-    <mergeCell ref="H18:I18"/>
-    <mergeCell ref="A19:B19"/>
-    <mergeCell ref="C19:D19"/>
-    <mergeCell ref="E19:G19"/>
-    <mergeCell ref="H19:I19"/>
-    <mergeCell ref="A16:B16"/>
-    <mergeCell ref="C16:D16"/>
-    <mergeCell ref="E16:G16"/>
-    <mergeCell ref="H16:I16"/>
-    <mergeCell ref="A17:B17"/>
-    <mergeCell ref="C17:D17"/>
-    <mergeCell ref="E17:G17"/>
-    <mergeCell ref="H17:I17"/>
-    <mergeCell ref="A14:B14"/>
-    <mergeCell ref="C14:D14"/>
-    <mergeCell ref="E14:G14"/>
-    <mergeCell ref="H14:I14"/>
-    <mergeCell ref="A15:B15"/>
-    <mergeCell ref="C15:D15"/>
-    <mergeCell ref="E15:G15"/>
-    <mergeCell ref="H15:I15"/>
-    <mergeCell ref="A12:B12"/>
-    <mergeCell ref="C12:D12"/>
-    <mergeCell ref="E12:G12"/>
-    <mergeCell ref="H12:I12"/>
-    <mergeCell ref="A13:B13"/>
-    <mergeCell ref="C13:D13"/>
-    <mergeCell ref="E13:G13"/>
-    <mergeCell ref="H13:I13"/>
-    <mergeCell ref="A10:B10"/>
-    <mergeCell ref="C10:D10"/>
-    <mergeCell ref="E10:G10"/>
-    <mergeCell ref="H10:I10"/>
-    <mergeCell ref="A11:B11"/>
-    <mergeCell ref="C11:D11"/>
-    <mergeCell ref="E11:G11"/>
-    <mergeCell ref="H11:I11"/>
-    <mergeCell ref="A1:I1"/>
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="C4:E4"/>
-    <mergeCell ref="F4:I4"/>
-    <mergeCell ref="A9:B9"/>
-    <mergeCell ref="C9:D9"/>
-    <mergeCell ref="E9:G9"/>
-    <mergeCell ref="H9:I9"/>
-    <mergeCell ref="A8:B8"/>
-    <mergeCell ref="C8:D8"/>
-    <mergeCell ref="D2:E2"/>
-    <mergeCell ref="E8:G8"/>
-    <mergeCell ref="H8:I8"/>
-    <mergeCell ref="F5:I5"/>
-    <mergeCell ref="A5:B5"/>
-    <mergeCell ref="C5:E5"/>
-    <mergeCell ref="B3:D3"/>
-  </mergeCells>
-  <printOptions gridLines="false" gridLinesSet="true"/>
-  <pageMargins left="0.70866141732283" right="0.51181102362205" top="0.74803149606299" bottom="0.74803149606299" header="0.31496062992126" footer="0.31496062992126"/>
-  <pageSetup paperSize="9" orientation="portrait" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" r:id="rId1ps"/>
+  <pageSetup paperSize="9" orientation="portrait" scale="100" fitToHeight="0" fitToWidth="0" pageOrder="downThenOver" r:id="rId1ps"/>
+  <rowBreaks count="1" manualBreakCount="1">
+    <brk id="25" man="1"/>
+  </rowBreaks>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Skladová karta: PDF pro WhatsApp (LibreOffice), oprava šablony.
Mobil sdílí PDF místo Excelu; token odkaz ke stažení; šablona z etalonu; LO scale 81 % pro 2× A4.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/deploy/excel/skladova-karta.template.xlsx
+++ b/deploy/excel/skladova-karta.template.xlsx
@@ -1,21 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xml:space="preserve">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
-  <workbookPr codeName="ThisWorkbook"/>
+  <workbookPr defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView activeTab="0" autoFilterDateGrouping="true" firstSheet="0" minimized="false" showHorizontalScroll="true" showSheetTabs="true" showVerticalScroll="true" tabRatio="600" visibility="visible"/>
+    <workbookView xWindow="120" yWindow="90" windowWidth="25815" windowHeight="11010"/>
   </bookViews>
   <sheets>
-    <sheet name="Skladová karta" sheetId="1" r:id="rId4"/>
+    <sheet name="Лист1" sheetId="1" r:id="rId1"/>
+    <sheet name="Лист2" sheetId="2" r:id="rId2"/>
+    <sheet name="Лист3" sheetId="3" r:id="rId3"/>
   </sheets>
-  <definedNames/>
-  <calcPr calcId="999999" calcMode="auto" calcCompleted="1" fullCalcOnLoad="0" forceFullCalc="0"/>
+  <calcPr calcId="124519"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="15">
   <si>
     <t>SKLADOVÁ KARTA - OPTIKA</t>
   </si>
@@ -23,22 +24,56 @@
     <t>DATUM NASKLADNĚNÍ :</t>
   </si>
   <si>
+    <t>CELKOVÁ METRÁŽ</t>
+  </si>
+  <si>
     <t>POČET VLÁKEN:</t>
+  </si>
+  <si>
+    <t>POČÁTEČNÍ STAV</t>
+  </si>
+  <si>
+    <t>TYP OK:</t>
+  </si>
+  <si>
+    <t>POZNÁMKA:</t>
   </si>
   <si>
     <t>ŠARŽE:</t>
   </si>
   <si>
-    <t>TYP OK:</t>
+    <t>450-020858</t>
   </si>
   <si>
-    <t>CELKOVÁ METRÁŽ</t>
+    <r>
+      <t xml:space="preserve">MLT  DROP  </t>
+    </r>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>BLOWN</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">  FLAT</t>
+    </r>
   </si>
   <si>
-    <t>POČÁTEČNÍ STAV</t>
-  </si>
-  <si>
-    <t>POZNÁMKA:</t>
+    <t>4 vl</t>
   </si>
   <si>
     <t>DATUM</t>
@@ -56,80 +91,103 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xml:space="preserve">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="_-* #,##0.00\ &quot;₴&quot;_-;\-* #,##0.00\ &quot;₴&quot;_-;_-* &quot;-&quot;??\ &quot;₴&quot;_-;_-@_-"/>
-    <numFmt numFmtId="165" formatCode="#,##0.0\ _₴"/>
+    <numFmt numFmtId="44" formatCode="_-* #,##0.00\ &quot;₴&quot;_-;\-* #,##0.00\ &quot;₴&quot;_-;_-* &quot;-&quot;??\ &quot;₴&quot;_-;_-@_-"/>
+    <numFmt numFmtId="164" formatCode="#,##0.0\ _₴"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="11">
     <font>
-      <b val="0"/>
-      <i val="0"/>
-      <strike val="0"/>
-      <u val="none"/>
       <sz val="11"/>
-      <color rgb="FF000000"/>
+      <color theme="1"/>
       <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="1"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b val="1"/>
-      <i val="0"/>
-      <strike val="0"/>
-      <u val="none"/>
-      <sz val="12"/>
-      <color rgb="FF000000"/>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="1"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b val="1"/>
-      <i val="0"/>
-      <strike val="0"/>
-      <u val="none"/>
-      <sz val="20"/>
-      <color rgb="FF000000"/>
+      <b/>
+      <sz val="18"/>
+      <color theme="1"/>
       <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="204"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b val="1"/>
-      <i val="0"/>
-      <strike val="0"/>
-      <u val="none"/>
-      <sz val="18"/>
-      <color rgb="FF000000"/>
+      <b/>
+      <sz val="20"/>
+      <color theme="1"/>
       <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="204"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b val="1"/>
-      <i val="0"/>
-      <strike val="0"/>
-      <u val="none"/>
+      <b/>
       <sz val="22"/>
-      <color rgb="FF000000"/>
+      <color theme="1"/>
       <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="204"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b val="0"/>
-      <i val="0"/>
-      <strike val="0"/>
-      <u val="none"/>
-      <sz val="13"/>
-      <color rgb="FF000000"/>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
       <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="204"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b val="0"/>
-      <i val="0"/>
-      <strike val="0"/>
-      <u val="none"/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="204"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="204"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="13"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="204"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <sz val="14"/>
-      <color rgb="FF000000"/>
+      <color theme="1"/>
       <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="204"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="14"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="1"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -142,8 +200,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFBFBFBF"/>
-        <bgColor rgb="FFFFFFFF"/>
+        <fgColor theme="0" tint="-0.249977111117893"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -156,43 +214,39 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
       <right/>
       <top style="thin">
-        <color rgb="FF000000"/>
+        <color indexed="64"/>
       </top>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
+      <bottom/>
       <diagonal/>
     </border>
     <border>
       <left/>
       <right/>
       <top style="thin">
-        <color rgb="FF000000"/>
+        <color indexed="64"/>
       </top>
-      <bottom style="medium">
-        <color rgb="FF000000"/>
-      </bottom>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
       <diagonal/>
     </border>
     <border>
       <left style="thin">
-        <color rgb="FF000000"/>
+        <color indexed="64"/>
       </left>
       <right/>
       <top/>
@@ -201,12 +255,12 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="FF000000"/>
+        <color indexed="64"/>
       </left>
       <right/>
       <top/>
       <bottom style="thin">
-        <color rgb="FF000000"/>
+        <color indexed="64"/>
       </bottom>
       <diagonal/>
     </border>
@@ -215,190 +269,196 @@
       <right/>
       <top/>
       <bottom style="thin">
-        <color rgb="FF000000"/>
+        <color indexed="64"/>
       </bottom>
       <diagonal/>
     </border>
     <border>
       <left/>
       <right style="thin">
-        <color rgb="FF000000"/>
+        <color indexed="64"/>
       </right>
       <top/>
       <bottom style="thin">
-        <color rgb="FF000000"/>
+        <color indexed="64"/>
       </bottom>
       <diagonal/>
     </border>
     <border>
       <left style="thin">
-        <color rgb="FF000000"/>
+        <color indexed="64"/>
       </left>
       <right/>
       <top style="thin">
-        <color rgb="FF000000"/>
+        <color indexed="64"/>
       </top>
-      <bottom/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
       <left/>
       <right/>
       <top style="thin">
-        <color rgb="FF000000"/>
+        <color indexed="64"/>
       </top>
-      <bottom/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
       <left/>
       <right style="thin">
-        <color rgb="FF000000"/>
+        <color indexed="64"/>
       </right>
       <top style="thin">
-        <color rgb="FF000000"/>
+        <color indexed="64"/>
       </top>
-      <bottom/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
+      <left/>
       <right/>
       <top style="thin">
-        <color rgb="FF000000"/>
+        <color indexed="64"/>
       </top>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
+      <bottom style="medium">
+        <color indexed="64"/>
       </bottom>
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="41">
-    <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="0" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
-    <xf xfId="0" fontId="0" numFmtId="164" fillId="0" borderId="0" applyFont="0" applyNumberFormat="1" applyFill="0" applyBorder="0" applyAlignment="0"/>
-    <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="0" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
-    <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="1" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="0"/>
-    <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="2" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="0"/>
-    <xf xfId="0" fontId="1" numFmtId="0" fillId="0" borderId="1" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
-    </xf>
-    <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="1" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
-    </xf>
-    <xf xfId="0" fontId="2" numFmtId="0" fillId="0" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
-    </xf>
-    <xf xfId="0" fontId="2" numFmtId="0" fillId="0" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="1">
-      <alignment vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
-    </xf>
-    <xf xfId="0" fontId="2" numFmtId="0" fillId="0" borderId="2" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
-    </xf>
-    <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="3" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="0"/>
-    <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="4" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="0"/>
-    <xf xfId="0" fontId="3" numFmtId="14" fillId="0" borderId="1" applyFont="1" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
-    </xf>
-    <xf xfId="0" fontId="3" numFmtId="14" fillId="0" borderId="2" applyFont="1" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
-    </xf>
-    <xf xfId="0" fontId="2" numFmtId="165" fillId="0" borderId="5" applyFont="1" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
-    </xf>
-    <xf xfId="0" fontId="2" numFmtId="165" fillId="0" borderId="6" applyFont="1" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
-    </xf>
-    <xf xfId="0" fontId="2" numFmtId="165" fillId="0" borderId="7" applyFont="1" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
-    </xf>
-    <xf xfId="0" fontId="3" numFmtId="0" fillId="0" borderId="5" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
-    </xf>
-    <xf xfId="0" fontId="3" numFmtId="0" fillId="0" borderId="7" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
-    </xf>
-    <xf xfId="0" fontId="2" numFmtId="0" fillId="0" borderId="5" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
-    </xf>
-    <xf xfId="0" fontId="2" numFmtId="0" fillId="0" borderId="6" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
-    </xf>
-    <xf xfId="0" fontId="2" numFmtId="0" fillId="0" borderId="7" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
-    </xf>
-    <xf xfId="0" fontId="2" numFmtId="0" fillId="0" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
-    </xf>
-    <xf xfId="0" fontId="4" numFmtId="164" fillId="0" borderId="0" applyFont="1" applyNumberFormat="1" applyFill="0" applyBorder="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
-    </xf>
-    <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="8" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="false" shrinkToFit="false"/>
-    </xf>
-    <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="9" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="false" shrinkToFit="false"/>
-    </xf>
-    <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="10" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="false" shrinkToFit="false"/>
-    </xf>
-    <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="4" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" shrinkToFit="false"/>
-    </xf>
-    <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="0" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" shrinkToFit="false"/>
-    </xf>
-    <xf xfId="0" fontId="0" numFmtId="0" fillId="2" borderId="4" applyFont="0" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" shrinkToFit="false"/>
-    </xf>
-    <xf xfId="0" fontId="0" numFmtId="0" fillId="2" borderId="0" applyFont="0" applyNumberFormat="0" applyFill="1" applyBorder="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" shrinkToFit="false"/>
-    </xf>
-    <xf xfId="0" fontId="5" numFmtId="0" fillId="0" borderId="11" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
-    </xf>
-    <xf xfId="0" fontId="5" numFmtId="0" fillId="0" borderId="5" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
-    </xf>
-    <xf xfId="0" fontId="5" numFmtId="0" fillId="0" borderId="8" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
-    </xf>
-    <xf xfId="0" fontId="5" numFmtId="0" fillId="0" borderId="10" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
-    </xf>
-    <xf xfId="0" fontId="5" numFmtId="0" fillId="0" borderId="11" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
-    </xf>
-    <xf xfId="0" fontId="5" numFmtId="0" fillId="0" borderId="9" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
-    </xf>
-    <xf xfId="0" fontId="6" numFmtId="0" fillId="2" borderId="4" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
-    </xf>
-    <xf xfId="0" fontId="6" numFmtId="0" fillId="2" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
-    </xf>
-    <xf xfId="0" fontId="6" numFmtId="0" fillId="2" borderId="4" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
-    </xf>
-    <xf xfId="0" fontId="6" numFmtId="0" fillId="2" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
-  <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+  <cellStyles count="2">
+    <cellStyle name="Денежный" xfId="1" builtinId="4"/>
+    <cellStyle name="Обычный" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotTableStyle1"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Тема Office">
   <a:themeElements>
     <a:clrScheme name="Стандартная">
       <a:dk1>
@@ -508,7 +568,7 @@
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Стандартная">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -681,25 +741,22 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xml:space="preserve" mc:Ignorable="x14ac">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:L48"/>
-  <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="9.28515625" customWidth="true" style="0"/>
-    <col min="2" max="2" width="10.28515625" customWidth="true" style="0"/>
-    <col min="4" max="4" width="13" customWidth="true" style="0"/>
-    <col min="5" max="5" width="7.28515625" customWidth="true" style="0"/>
-    <col min="6" max="6" width="9.28515625" customWidth="true" style="0"/>
-    <col min="7" max="7" width="6.7109375" customWidth="true" style="0"/>
-    <col min="8" max="8" width="6.85546875" customWidth="true" style="0"/>
-    <col min="9" max="9" width="16.42578125" customWidth="true" style="0"/>
-    <col min="10" max="10" width="1" customWidth="true" style="0"/>
+    <col min="1" max="1" width="9.28515625" customWidth="1"/>
+    <col min="2" max="2" width="10.28515625" customWidth="1"/>
+    <col min="4" max="4" width="13" customWidth="1"/>
+    <col min="5" max="5" width="7.28515625" customWidth="1"/>
+    <col min="6" max="6" width="9.28515625" customWidth="1"/>
+    <col min="7" max="7" width="6.7109375" customWidth="1"/>
+    <col min="8" max="8" width="6.85546875" customWidth="1"/>
+    <col min="9" max="9" width="16.42578125" customWidth="1"/>
+    <col min="10" max="10" width="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" customHeight="1" ht="28.5">
+    <row r="1" spans="1:12" ht="28.5">
       <c r="A1" s="23" t="s">
         <v>0</v>
       </c>
@@ -715,68 +772,82 @@
       <c r="K1" s="1"/>
       <c r="L1" s="1"/>
     </row>
-    <row r="2" spans="1:12" customHeight="1" ht="33">
+    <row r="2" spans="1:12" ht="33" customHeight="1">
       <c r="A2" s="31" t="s">
         <v>1</v>
       </c>
       <c r="B2" s="3"/>
       <c r="C2" s="3"/>
-      <c r="D2" s="12"/>
+      <c r="D2" s="12">
+        <v>46167</v>
+      </c>
       <c r="E2" s="13"/>
       <c r="F2" s="31" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G2" s="5"/>
       <c r="H2" s="3"/>
-      <c r="I2" s="9"/>
+      <c r="I2" s="9" t="s">
+        <v>10</v>
+      </c>
       <c r="J2" s="8"/>
       <c r="K2" s="8"/>
     </row>
-    <row r="3" spans="1:12" customHeight="1" ht="33.75">
+    <row r="3" spans="1:12" ht="33.75" customHeight="1">
       <c r="A3" s="32" t="s">
-        <v>3</v>
-      </c>
-      <c r="B3" s="22"/>
+        <v>7</v>
+      </c>
+      <c r="B3" s="22" t="s">
+        <v>8</v>
+      </c>
       <c r="C3" s="22"/>
       <c r="D3" s="22"/>
       <c r="E3" s="7"/>
       <c r="F3" s="35" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G3" s="5"/>
-      <c r="H3" s="6"/>
+      <c r="H3" s="6" t="s">
+        <v>9</v>
+      </c>
       <c r="I3" s="4"/>
       <c r="J3" s="11"/>
     </row>
-    <row r="4" spans="1:12" customHeight="1" ht="26.25">
+    <row r="4" spans="1:12" ht="26.25" customHeight="1">
       <c r="A4" s="33" t="s">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="B4" s="34"/>
       <c r="C4" s="33" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D4" s="36"/>
       <c r="E4" s="34"/>
       <c r="F4" s="24" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G4" s="25"/>
       <c r="H4" s="25"/>
       <c r="I4" s="26"/>
     </row>
-    <row r="5" spans="1:12" customHeight="1" ht="35.25">
-      <c r="A5" s="17"/>
+    <row r="5" spans="1:12" ht="35.25" customHeight="1">
+      <c r="A5" s="17">
+        <v>2100</v>
+      </c>
       <c r="B5" s="18"/>
-      <c r="C5" s="19"/>
+      <c r="C5" s="19">
+        <v>4500</v>
+      </c>
       <c r="D5" s="20"/>
       <c r="E5" s="21"/>
-      <c r="F5" s="14"/>
+      <c r="F5" s="14">
+        <v>2</v>
+      </c>
       <c r="G5" s="15"/>
       <c r="H5" s="15"/>
       <c r="I5" s="16"/>
     </row>
-    <row r="6" spans="1:12" customHeight="1" ht="9">
+    <row r="6" spans="1:12" ht="9" customHeight="1" thickBot="1">
       <c r="A6" s="10"/>
       <c r="B6" s="10"/>
       <c r="C6" s="10"/>
@@ -787,30 +858,30 @@
       <c r="H6" s="10"/>
       <c r="I6" s="10"/>
     </row>
-    <row r="7" spans="1:12" customHeight="1" ht="12">
+    <row r="7" spans="1:12" ht="12" customHeight="1">
       <c r="I7" s="2"/>
     </row>
-    <row r="8" spans="1:12" customHeight="1" ht="32.1">
+    <row r="8" spans="1:12" ht="32.1" customHeight="1">
       <c r="A8" s="39" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="B8" s="40"/>
       <c r="C8" s="37" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="D8" s="38"/>
       <c r="E8" s="37" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="F8" s="38"/>
       <c r="G8" s="38"/>
       <c r="H8" s="37" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="I8" s="38"/>
       <c r="J8" s="11"/>
     </row>
-    <row r="9" spans="1:12" customHeight="1" ht="32.1">
+    <row r="9" spans="1:12" ht="32.1" customHeight="1">
       <c r="A9" s="27"/>
       <c r="B9" s="28"/>
       <c r="C9" s="27"/>
@@ -822,7 +893,7 @@
       <c r="I9" s="28"/>
       <c r="J9" s="11"/>
     </row>
-    <row r="10" spans="1:12" customHeight="1" ht="32.1">
+    <row r="10" spans="1:12" ht="32.1" customHeight="1">
       <c r="A10" s="29"/>
       <c r="B10" s="30"/>
       <c r="C10" s="29"/>
@@ -834,7 +905,7 @@
       <c r="I10" s="30"/>
       <c r="J10" s="11"/>
     </row>
-    <row r="11" spans="1:12" customHeight="1" ht="32.1">
+    <row r="11" spans="1:12" ht="32.1" customHeight="1">
       <c r="A11" s="27"/>
       <c r="B11" s="28"/>
       <c r="C11" s="27"/>
@@ -846,7 +917,7 @@
       <c r="I11" s="28"/>
       <c r="J11" s="11"/>
     </row>
-    <row r="12" spans="1:12" customHeight="1" ht="32.1">
+    <row r="12" spans="1:12" ht="32.1" customHeight="1">
       <c r="A12" s="29"/>
       <c r="B12" s="30"/>
       <c r="C12" s="29"/>
@@ -858,7 +929,7 @@
       <c r="I12" s="30"/>
       <c r="J12" s="11"/>
     </row>
-    <row r="13" spans="1:12" customHeight="1" ht="32.1">
+    <row r="13" spans="1:12" ht="32.1" customHeight="1">
       <c r="A13" s="27"/>
       <c r="B13" s="28"/>
       <c r="C13" s="27"/>
@@ -870,7 +941,7 @@
       <c r="I13" s="28"/>
       <c r="J13" s="11"/>
     </row>
-    <row r="14" spans="1:12" customHeight="1" ht="32.1">
+    <row r="14" spans="1:12" ht="32.1" customHeight="1">
       <c r="A14" s="29"/>
       <c r="B14" s="30"/>
       <c r="C14" s="29"/>
@@ -882,7 +953,7 @@
       <c r="I14" s="30"/>
       <c r="J14" s="11"/>
     </row>
-    <row r="15" spans="1:12" customHeight="1" ht="32.1">
+    <row r="15" spans="1:12" ht="32.1" customHeight="1">
       <c r="A15" s="27"/>
       <c r="B15" s="28"/>
       <c r="C15" s="27"/>
@@ -894,7 +965,7 @@
       <c r="I15" s="28"/>
       <c r="J15" s="11"/>
     </row>
-    <row r="16" spans="1:12" customHeight="1" ht="32.1">
+    <row r="16" spans="1:12" ht="32.1" customHeight="1">
       <c r="A16" s="29"/>
       <c r="B16" s="30"/>
       <c r="C16" s="29"/>
@@ -906,7 +977,7 @@
       <c r="I16" s="30"/>
       <c r="J16" s="11"/>
     </row>
-    <row r="17" spans="1:12" customHeight="1" ht="32.1">
+    <row r="17" spans="1:10" ht="32.1" customHeight="1">
       <c r="A17" s="27"/>
       <c r="B17" s="28"/>
       <c r="C17" s="27"/>
@@ -918,7 +989,7 @@
       <c r="I17" s="28"/>
       <c r="J17" s="11"/>
     </row>
-    <row r="18" spans="1:12" customHeight="1" ht="32.1">
+    <row r="18" spans="1:10" ht="32.1" customHeight="1">
       <c r="A18" s="29"/>
       <c r="B18" s="30"/>
       <c r="C18" s="29"/>
@@ -930,7 +1001,7 @@
       <c r="I18" s="30"/>
       <c r="J18" s="11"/>
     </row>
-    <row r="19" spans="1:12" customHeight="1" ht="32.1">
+    <row r="19" spans="1:10" ht="32.1" customHeight="1">
       <c r="A19" s="27"/>
       <c r="B19" s="28"/>
       <c r="C19" s="27"/>
@@ -942,7 +1013,7 @@
       <c r="I19" s="28"/>
       <c r="J19" s="11"/>
     </row>
-    <row r="20" spans="1:12" customHeight="1" ht="32.1">
+    <row r="20" spans="1:10" ht="32.1" customHeight="1">
       <c r="A20" s="29"/>
       <c r="B20" s="30"/>
       <c r="C20" s="29"/>
@@ -954,7 +1025,7 @@
       <c r="I20" s="30"/>
       <c r="J20" s="11"/>
     </row>
-    <row r="21" spans="1:12" customHeight="1" ht="32.1">
+    <row r="21" spans="1:10" ht="32.1" customHeight="1">
       <c r="A21" s="27"/>
       <c r="B21" s="28"/>
       <c r="C21" s="27"/>
@@ -966,7 +1037,7 @@
       <c r="I21" s="28"/>
       <c r="J21" s="11"/>
     </row>
-    <row r="22" spans="1:12" customHeight="1" ht="32.1">
+    <row r="22" spans="1:10" ht="32.1" customHeight="1">
       <c r="A22" s="29"/>
       <c r="B22" s="30"/>
       <c r="C22" s="29"/>
@@ -978,7 +1049,7 @@
       <c r="I22" s="30"/>
       <c r="J22" s="11"/>
     </row>
-    <row r="23" spans="1:12" customHeight="1" ht="32.1">
+    <row r="23" spans="1:10" ht="32.1" customHeight="1">
       <c r="A23" s="27"/>
       <c r="B23" s="28"/>
       <c r="C23" s="27"/>
@@ -990,7 +1061,7 @@
       <c r="I23" s="28"/>
       <c r="J23" s="11"/>
     </row>
-    <row r="24" spans="1:12" customHeight="1" ht="32.1">
+    <row r="24" spans="1:10" ht="32.1" customHeight="1">
       <c r="A24" s="29"/>
       <c r="B24" s="30"/>
       <c r="C24" s="29"/>
@@ -1002,7 +1073,7 @@
       <c r="I24" s="30"/>
       <c r="J24" s="11"/>
     </row>
-    <row r="25" spans="1:12" customHeight="1" ht="32.1">
+    <row r="25" spans="1:10" ht="32.1" customHeight="1">
       <c r="A25" s="27"/>
       <c r="B25" s="28"/>
       <c r="C25" s="27"/>
@@ -1014,27 +1085,27 @@
       <c r="I25" s="28"/>
       <c r="J25" s="11"/>
     </row>
-    <row r="26" spans="1:12" customHeight="1" ht="32.1">
+    <row r="26" spans="1:10" ht="32.1" customHeight="1">
       <c r="A26" s="37" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="B26" s="38"/>
       <c r="C26" s="37" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="D26" s="38"/>
       <c r="E26" s="37" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="F26" s="38"/>
       <c r="G26" s="38"/>
       <c r="H26" s="37" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="I26" s="38"/>
       <c r="J26" s="11"/>
     </row>
-    <row r="27" spans="1:12" customHeight="1" ht="32.1">
+    <row r="27" spans="1:10" ht="32.1" customHeight="1">
       <c r="A27" s="27"/>
       <c r="B27" s="28"/>
       <c r="C27" s="27"/>
@@ -1046,7 +1117,7 @@
       <c r="I27" s="28"/>
       <c r="J27" s="11"/>
     </row>
-    <row r="28" spans="1:12" customHeight="1" ht="32.1">
+    <row r="28" spans="1:10" ht="32.1" customHeight="1">
       <c r="A28" s="29"/>
       <c r="B28" s="30"/>
       <c r="C28" s="29"/>
@@ -1058,7 +1129,7 @@
       <c r="I28" s="30"/>
       <c r="J28" s="11"/>
     </row>
-    <row r="29" spans="1:12" customHeight="1" ht="32.1">
+    <row r="29" spans="1:10" ht="32.1" customHeight="1">
       <c r="A29" s="27"/>
       <c r="B29" s="28"/>
       <c r="C29" s="27"/>
@@ -1070,7 +1141,7 @@
       <c r="I29" s="28"/>
       <c r="J29" s="11"/>
     </row>
-    <row r="30" spans="1:12" customHeight="1" ht="32.1">
+    <row r="30" spans="1:10" ht="32.1" customHeight="1">
       <c r="A30" s="29"/>
       <c r="B30" s="30"/>
       <c r="C30" s="29"/>
@@ -1082,7 +1153,7 @@
       <c r="I30" s="30"/>
       <c r="J30" s="11"/>
     </row>
-    <row r="31" spans="1:12" customHeight="1" ht="32.1">
+    <row r="31" spans="1:10" ht="32.1" customHeight="1">
       <c r="A31" s="27"/>
       <c r="B31" s="28"/>
       <c r="C31" s="27"/>
@@ -1094,7 +1165,7 @@
       <c r="I31" s="28"/>
       <c r="J31" s="11"/>
     </row>
-    <row r="32" spans="1:12" customHeight="1" ht="32.1">
+    <row r="32" spans="1:10" ht="32.1" customHeight="1">
       <c r="A32" s="29"/>
       <c r="B32" s="30"/>
       <c r="C32" s="29"/>
@@ -1106,7 +1177,7 @@
       <c r="I32" s="30"/>
       <c r="J32" s="11"/>
     </row>
-    <row r="33" spans="1:12" customHeight="1" ht="32.1">
+    <row r="33" spans="1:10" ht="32.1" customHeight="1">
       <c r="A33" s="27"/>
       <c r="B33" s="28"/>
       <c r="C33" s="27"/>
@@ -1118,7 +1189,7 @@
       <c r="I33" s="28"/>
       <c r="J33" s="11"/>
     </row>
-    <row r="34" spans="1:12" customHeight="1" ht="32.1">
+    <row r="34" spans="1:10" ht="32.1" customHeight="1">
       <c r="A34" s="29"/>
       <c r="B34" s="30"/>
       <c r="C34" s="29"/>
@@ -1130,7 +1201,7 @@
       <c r="I34" s="30"/>
       <c r="J34" s="11"/>
     </row>
-    <row r="35" spans="1:12" customHeight="1" ht="32.1">
+    <row r="35" spans="1:10" ht="32.1" customHeight="1">
       <c r="A35" s="27"/>
       <c r="B35" s="28"/>
       <c r="C35" s="27"/>
@@ -1142,7 +1213,7 @@
       <c r="I35" s="28"/>
       <c r="J35" s="11"/>
     </row>
-    <row r="36" spans="1:12" customHeight="1" ht="32.1">
+    <row r="36" spans="1:10" ht="32.1" customHeight="1">
       <c r="A36" s="29"/>
       <c r="B36" s="30"/>
       <c r="C36" s="29"/>
@@ -1154,7 +1225,7 @@
       <c r="I36" s="30"/>
       <c r="J36" s="11"/>
     </row>
-    <row r="37" spans="1:12" customHeight="1" ht="32.1">
+    <row r="37" spans="1:10" ht="32.1" customHeight="1">
       <c r="A37" s="27"/>
       <c r="B37" s="28"/>
       <c r="C37" s="27"/>
@@ -1166,7 +1237,7 @@
       <c r="I37" s="28"/>
       <c r="J37" s="11"/>
     </row>
-    <row r="38" spans="1:12" customHeight="1" ht="32.1">
+    <row r="38" spans="1:10" ht="32.1" customHeight="1">
       <c r="A38" s="29"/>
       <c r="B38" s="30"/>
       <c r="C38" s="29"/>
@@ -1178,7 +1249,7 @@
       <c r="I38" s="30"/>
       <c r="J38" s="11"/>
     </row>
-    <row r="39" spans="1:12" customHeight="1" ht="32.1">
+    <row r="39" spans="1:10" ht="32.1" customHeight="1">
       <c r="A39" s="27"/>
       <c r="B39" s="28"/>
       <c r="C39" s="27"/>
@@ -1190,7 +1261,7 @@
       <c r="I39" s="28"/>
       <c r="J39" s="11"/>
     </row>
-    <row r="40" spans="1:12" customHeight="1" ht="32.1">
+    <row r="40" spans="1:10" ht="32.1" customHeight="1">
       <c r="A40" s="29"/>
       <c r="B40" s="30"/>
       <c r="C40" s="29"/>
@@ -1202,7 +1273,7 @@
       <c r="I40" s="30"/>
       <c r="J40" s="11"/>
     </row>
-    <row r="41" spans="1:12" customHeight="1" ht="32.1">
+    <row r="41" spans="1:10" ht="32.1" customHeight="1">
       <c r="A41" s="27"/>
       <c r="B41" s="28"/>
       <c r="C41" s="27"/>
@@ -1214,7 +1285,7 @@
       <c r="I41" s="28"/>
       <c r="J41" s="11"/>
     </row>
-    <row r="42" spans="1:12" customHeight="1" ht="32.1">
+    <row r="42" spans="1:10" ht="32.1" customHeight="1">
       <c r="A42" s="29"/>
       <c r="B42" s="30"/>
       <c r="C42" s="29"/>
@@ -1226,7 +1297,7 @@
       <c r="I42" s="30"/>
       <c r="J42" s="11"/>
     </row>
-    <row r="43" spans="1:12" customHeight="1" ht="32.1">
+    <row r="43" spans="1:10" ht="32.1" customHeight="1">
       <c r="A43" s="27"/>
       <c r="B43" s="28"/>
       <c r="C43" s="27"/>
@@ -1238,7 +1309,7 @@
       <c r="I43" s="28"/>
       <c r="J43" s="11"/>
     </row>
-    <row r="44" spans="1:12" customHeight="1" ht="32.1">
+    <row r="44" spans="1:10" ht="32.1" customHeight="1">
       <c r="A44" s="29"/>
       <c r="B44" s="30"/>
       <c r="C44" s="29"/>
@@ -1250,7 +1321,7 @@
       <c r="I44" s="30"/>
       <c r="J44" s="11"/>
     </row>
-    <row r="45" spans="1:12" customHeight="1" ht="32.1">
+    <row r="45" spans="1:10" ht="32.1" customHeight="1">
       <c r="A45" s="27"/>
       <c r="B45" s="28"/>
       <c r="C45" s="27"/>
@@ -1262,7 +1333,7 @@
       <c r="I45" s="28"/>
       <c r="J45" s="11"/>
     </row>
-    <row r="46" spans="1:12" customHeight="1" ht="32.1">
+    <row r="46" spans="1:10" ht="32.1" customHeight="1">
       <c r="A46" s="29"/>
       <c r="B46" s="30"/>
       <c r="C46" s="29"/>
@@ -1274,7 +1345,7 @@
       <c r="I46" s="30"/>
       <c r="J46" s="11"/>
     </row>
-    <row r="47" spans="1:12" customHeight="1" ht="32.1">
+    <row r="47" spans="1:10" ht="32.1" customHeight="1">
       <c r="A47" s="27"/>
       <c r="B47" s="28"/>
       <c r="C47" s="27"/>
@@ -1286,7 +1357,7 @@
       <c r="I47" s="28"/>
       <c r="J47" s="11"/>
     </row>
-    <row r="48" spans="1:12" customHeight="1" ht="32.1">
+    <row r="48" spans="1:10" ht="32.1" customHeight="1">
       <c r="A48" s="29"/>
       <c r="B48" s="30"/>
       <c r="C48" s="29"/>
@@ -1299,7 +1370,7 @@
       <c r="J48" s="11"/>
     </row>
   </sheetData>
-  <mergeCells>
+  <mergeCells count="173">
     <mergeCell ref="A48:B48"/>
     <mergeCell ref="C48:D48"/>
     <mergeCell ref="E48:G48"/>
@@ -1474,11 +1545,28 @@
     <mergeCell ref="C5:E5"/>
     <mergeCell ref="B3:D3"/>
   </mergeCells>
-  <printOptions gridLines="false" gridLinesSet="true"/>
-  <pageMargins left="0.70866141732283" right="0.51181102362205" top="0.74803149606299" bottom="0.74803149606299" header="0.31496062992126" footer="0.31496062992126"/>
-  <pageSetup paperSize="9" orientation="portrait" scale="100" fitToHeight="0" fitToWidth="0" pageOrder="downThenOver" r:id="rId1ps"/>
+  <pageMargins left="0.70866141732283472" right="0.51181102362204722" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
+  <pageSetup paperSize="9" orientation="portrait" scale="100" fitToHeight="0" fitToWidth="0" pageOrder="downThenOver"/>
   <rowBreaks count="1" manualBreakCount="1">
     <brk id="25" man="1"/>
   </rowBreaks>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>